<commit_message>
1.0.1 - personal information
</commit_message>
<xml_diff>
--- a/function/menu_CsvMaker_v2.xlsx
+++ b/function/menu_CsvMaker_v2.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\utmassetx\function\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\assetx\function\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDDC451E-0C65-4444-AA20-D588BB335856}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4B39343-DD21-4328-AE77-FDE823E74893}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9BC57BCF-AE79-4796-BD03-06513ABF4AED}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1076" uniqueCount="233">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1156" uniqueCount="252">
   <si>
     <t>filename</t>
   </si>
@@ -735,6 +735,63 @@
   <si>
     <t>subpages/formv1/formv1jabatan.dat</t>
   </si>
+  <si>
+    <t>Profile</t>
+  </si>
+  <si>
+    <t>Personal</t>
+  </si>
+  <si>
+    <t>Account &amp; Security</t>
+  </si>
+  <si>
+    <t>Privacy</t>
+  </si>
+  <si>
+    <t>Account</t>
+  </si>
+  <si>
+    <t>Password</t>
+  </si>
+  <si>
+    <t>Two-Factor Authentication</t>
+  </si>
+  <si>
+    <t>Active Sessions</t>
+  </si>
+  <si>
+    <t>Login History</t>
+  </si>
+  <si>
+    <t>file107</t>
+  </si>
+  <si>
+    <t>file109</t>
+  </si>
+  <si>
+    <t>file110</t>
+  </si>
+  <si>
+    <t>file111</t>
+  </si>
+  <si>
+    <t>file112</t>
+  </si>
+  <si>
+    <t>file113</t>
+  </si>
+  <si>
+    <t>file114</t>
+  </si>
+  <si>
+    <t>file115</t>
+  </si>
+  <si>
+    <t>file116</t>
+  </si>
+  <si>
+    <t>subpages/profile/personal/personal.php</t>
+  </si>
 </sst>
 </file>
 
@@ -891,9 +948,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -931,7 +988,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1037,7 +1094,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1179,7 +1236,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1187,7 +1244,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53E3E82A-C4E5-4D71-9206-9534853B9196}">
-  <dimension ref="B11:DL118"/>
+  <dimension ref="B11:DL128"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="31" width="3.140625" customWidth="1"/>
@@ -25915,7 +25972,7 @@
         <v>066</v>
       </c>
       <c r="CF78" t="str">
-        <f t="shared" ref="CF78:CH118" si="181">TEXT(0,"00")</f>
+        <f t="shared" ref="CF78:CH119" si="181">TEXT(0,"00")</f>
         <v>00</v>
       </c>
       <c r="CG78" t="str">
@@ -26042,7 +26099,7 @@
     </row>
     <row r="79" spans="2:116" x14ac:dyDescent="0.25">
       <c r="B79">
-        <f t="shared" ref="B79:B118" si="205">B78+1</f>
+        <f t="shared" ref="B79:B131" si="205">B78+1</f>
         <v>67</v>
       </c>
       <c r="F79" t="s">
@@ -40838,6 +40895,3706 @@
       <c r="DL118" t="str">
         <f t="shared" si="204"/>
         <v>106,00,00,00,01,06,03,04,00,00,00,00,00,00,00,00,00,00,00,00,00,00,00,04,0106030400000000000000000000000000000004,Delete aku,file106,Blk1,Blk2,Blk3,Blk4,Blk5,Blk6</v>
+      </c>
+    </row>
+    <row r="119" spans="2:116" x14ac:dyDescent="0.25">
+      <c r="B119">
+        <f t="shared" si="205"/>
+        <v>107</v>
+      </c>
+      <c r="D119" t="s">
+        <v>233</v>
+      </c>
+      <c r="W119">
+        <f t="shared" ref="W119:W128" si="244">IF(C119&lt;&gt;"",1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="X119">
+        <f t="shared" ref="X119:X128" si="245">IF(D119&lt;&gt;"",1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="Y119">
+        <f t="shared" ref="Y119:Y128" si="246">IF(E119&lt;&gt;"",1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="Z119">
+        <f t="shared" ref="Z119:Z128" si="247">IF(F119&lt;&gt;"",1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="AA119">
+        <f t="shared" ref="AA119:AA128" si="248">IF(G119&lt;&gt;"",1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="AB119">
+        <f t="shared" ref="AB119:AB128" si="249">IF(H119&lt;&gt;"",1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="AC119">
+        <f t="shared" ref="AC119:AC128" si="250">IF(I119&lt;&gt;"",1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="AD119">
+        <f t="shared" ref="AD119:AD128" si="251">IF(J119&lt;&gt;"",1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="AE119">
+        <f t="shared" ref="AE119:AE128" si="252">IF(K119&lt;&gt;"",1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="AF119">
+        <f t="shared" ref="AF119:AF128" si="253">IF(L119&lt;&gt;"",1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="AG119">
+        <f t="shared" ref="AG119:AG128" si="254">IF(M119&lt;&gt;"",1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="AH119">
+        <f t="shared" ref="AH119:AH128" si="255">IF(N119&lt;&gt;"",1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="AI119">
+        <f t="shared" ref="AI119:AI128" si="256">IF(O119&lt;&gt;"",1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="AJ119">
+        <f t="shared" ref="AJ119:AJ128" si="257">IF(P119&lt;&gt;"",1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="AK119">
+        <f t="shared" ref="AK119:AK128" si="258">IF(Q119&lt;&gt;"",1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="AL119">
+        <f t="shared" ref="AL119:AL128" si="259">IF(R119&lt;&gt;"",1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="AM119">
+        <f t="shared" ref="AM119:AM128" si="260">IF(S119&lt;&gt;"",1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="AN119">
+        <f t="shared" ref="AN119:AN128" si="261">IF(T119&lt;&gt;"",1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="AO119">
+        <f t="shared" ref="AO119:AO128" si="262">IF(U119&lt;&gt;"",1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="AP119" s="2" t="str">
+        <f t="shared" ref="AP119:AP128" si="263">IF(SUM(W119:AO119)&gt;1,"Error","")</f>
+        <v/>
+      </c>
+      <c r="AQ119" t="str">
+        <f t="shared" ref="AQ119:AQ128" si="264">IF(AND(W119=1,W118=1),"+",IF(AND(W119=1,W118=0),IF(AQ118="S","+",1),IF(AND(AQ118&lt;&gt;"",AR119&lt;&gt;""),"S","")))</f>
+        <v>S</v>
+      </c>
+      <c r="AR119" t="str">
+        <f t="shared" ref="AR119:AR128" si="265">IF(AND(X119=1,X118=1),"+",IF(AND(X119=1,X118=0),IF(AR118="S","+",1),IF(AND(AR118&lt;&gt;"",AS119&lt;&gt;""),"S","")))</f>
+        <v>+</v>
+      </c>
+      <c r="AS119" t="str">
+        <f t="shared" ref="AS119:AS128" si="266">IF(AND(Y119=1,Y118=1),"+",IF(AND(Y119=1,Y118=0),IF(AS118="S","+",1),IF(AND(AS118&lt;&gt;"",AT119&lt;&gt;""),"S","")))</f>
+        <v/>
+      </c>
+      <c r="AT119" t="str">
+        <f t="shared" ref="AT119:AT128" si="267">IF(AND(Z119=1,Z118=1),"+",IF(AND(Z119=1,Z118=0),IF(AT118="S","+",1),IF(AND(AT118&lt;&gt;"",AU119&lt;&gt;""),"S","")))</f>
+        <v/>
+      </c>
+      <c r="AU119" t="str">
+        <f t="shared" ref="AU119:AU128" si="268">IF(AND(AA119=1,AA118=1),"+",IF(AND(AA119=1,AA118=0),IF(AU118="S","+",1),IF(AND(AU118&lt;&gt;"",AV119&lt;&gt;""),"S","")))</f>
+        <v/>
+      </c>
+      <c r="AV119" t="str">
+        <f t="shared" ref="AV119:AV128" si="269">IF(AND(AB119=1,AB118=1),"+",IF(AND(AB119=1,AB118=0),IF(AV118="S","+",1),IF(AND(AV118&lt;&gt;"",AW119&lt;&gt;""),"S","")))</f>
+        <v/>
+      </c>
+      <c r="AW119" t="str">
+        <f t="shared" ref="AW119:AW128" si="270">IF(AND(AC119=1,AC118=1),"+",IF(AND(AC119=1,AC118=0),IF(AW118="S","+",1),IF(AND(AW118&lt;&gt;"",AX119&lt;&gt;""),"S","")))</f>
+        <v/>
+      </c>
+      <c r="AX119" t="str">
+        <f t="shared" ref="AX119:AX128" si="271">IF(AND(AD119=1,AD118=1),"+",IF(AND(AD119=1,AD118=0),IF(AX118="S","+",1),IF(AND(AX118&lt;&gt;"",AY119&lt;&gt;""),"S","")))</f>
+        <v/>
+      </c>
+      <c r="AY119" t="str">
+        <f t="shared" ref="AY119:AY128" si="272">IF(AND(AE119=1,AE118=1),"+",IF(AND(AE119=1,AE118=0),IF(AY118="S","+",1),IF(AND(AY118&lt;&gt;"",AZ119&lt;&gt;""),"S","")))</f>
+        <v/>
+      </c>
+      <c r="AZ119" t="str">
+        <f t="shared" ref="AZ119:AZ128" si="273">IF(AND(AF119=1,AF118=1),"+",IF(AND(AF119=1,AF118=0),IF(AZ118="S","+",1),IF(AND(AZ118&lt;&gt;"",BA119&lt;&gt;""),"S","")))</f>
+        <v/>
+      </c>
+      <c r="BA119" t="str">
+        <f t="shared" ref="BA119:BA128" si="274">IF(AND(AG119=1,AG118=1),"+",IF(AND(AG119=1,AG118=0),IF(BA118="S","+",1),IF(AND(BA118&lt;&gt;"",BB119&lt;&gt;""),"S","")))</f>
+        <v/>
+      </c>
+      <c r="BB119" t="str">
+        <f t="shared" ref="BB119:BB128" si="275">IF(AND(AH119=1,AH118=1),"+",IF(AND(AH119=1,AH118=0),IF(BB118="S","+",1),IF(AND(BB118&lt;&gt;"",BC119&lt;&gt;""),"S","")))</f>
+        <v/>
+      </c>
+      <c r="BC119" t="str">
+        <f t="shared" ref="BC119:BC128" si="276">IF(AND(AI119=1,AI118=1),"+",IF(AND(AI119=1,AI118=0),IF(BC118="S","+",1),IF(AND(BC118&lt;&gt;"",BD119&lt;&gt;""),"S","")))</f>
+        <v/>
+      </c>
+      <c r="BD119" t="str">
+        <f t="shared" ref="BD119:BD128" si="277">IF(AND(AJ119=1,AJ118=1),"+",IF(AND(AJ119=1,AJ118=0),IF(BD118="S","+",1),IF(AND(BD118&lt;&gt;"",BE119&lt;&gt;""),"S","")))</f>
+        <v/>
+      </c>
+      <c r="BE119" t="str">
+        <f t="shared" ref="BE119:BE128" si="278">IF(AND(AK119=1,AK118=1),"+",IF(AND(AK119=1,AK118=0),IF(BE118="S","+",1),IF(AND(BE118&lt;&gt;"",BF119&lt;&gt;""),"S","")))</f>
+        <v/>
+      </c>
+      <c r="BF119" t="str">
+        <f t="shared" ref="BF119:BF128" si="279">IF(AND(AL119=1,AL118=1),"+",IF(AND(AL119=1,AL118=0),IF(BF118="S","+",1),IF(AND(BF118&lt;&gt;"",BG119&lt;&gt;""),"S","")))</f>
+        <v/>
+      </c>
+      <c r="BG119" t="str">
+        <f t="shared" ref="BG119:BG128" si="280">IF(AND(AM119=1,AM118=1),"+",IF(AND(AM119=1,AM118=0),IF(BG118="S","+",1),IF(AND(BG118&lt;&gt;"",BH119&lt;&gt;""),"S","")))</f>
+        <v/>
+      </c>
+      <c r="BH119" t="str">
+        <f t="shared" ref="BH119:BH128" si="281">IF(AND(AN119=1,AN118=1),"+",IF(AND(AN119=1,AN118=0),IF(BH118="S","+",1),IF(AND(BH118&lt;&gt;"",BI119&lt;&gt;""),"S","")))</f>
+        <v/>
+      </c>
+      <c r="BI119" t="str">
+        <f t="shared" ref="BI119:BI128" si="282">IF(AND(AO119=1,AO118=1),"+",IF(AND(AO119=1,AO118=0),IF(BI118="S","+",1),IF(AND(BI118&lt;&gt;"",BJ119&lt;&gt;""),"S","")))</f>
+        <v/>
+      </c>
+      <c r="BK119">
+        <f t="shared" ref="BK119:BK128" si="283">IF(AQ119=1,1,IF(AQ119="S",BK118,IF(AQ119="+",BK118+1,0)))</f>
+        <v>1</v>
+      </c>
+      <c r="BL119">
+        <f t="shared" ref="BL119:BL128" si="284">IF(AR119=1,1,IF(AR119="S",BL118,IF(AR119="+",BL118+1,0)))</f>
+        <v>7</v>
+      </c>
+      <c r="BM119">
+        <f t="shared" ref="BM119:BM128" si="285">IF(AS119=1,1,IF(AS119="S",BM118,IF(AS119="+",BM118+1,0)))</f>
+        <v>0</v>
+      </c>
+      <c r="BN119">
+        <f t="shared" ref="BN119:BN128" si="286">IF(AT119=1,1,IF(AT119="S",BN118,IF(AT119="+",BN118+1,0)))</f>
+        <v>0</v>
+      </c>
+      <c r="BO119">
+        <f t="shared" ref="BO119:BO128" si="287">IF(AU119=1,1,IF(AU119="S",BO118,IF(AU119="+",BO118+1,0)))</f>
+        <v>0</v>
+      </c>
+      <c r="BP119">
+        <f t="shared" ref="BP119:BP128" si="288">IF(AV119=1,1,IF(AV119="S",BP118,IF(AV119="+",BP118+1,0)))</f>
+        <v>0</v>
+      </c>
+      <c r="BQ119">
+        <f t="shared" ref="BQ119:BQ128" si="289">IF(AW119=1,1,IF(AW119="S",BQ118,IF(AW119="+",BQ118+1,0)))</f>
+        <v>0</v>
+      </c>
+      <c r="BR119">
+        <f t="shared" ref="BR119:BR128" si="290">IF(AX119=1,1,IF(AX119="S",BR118,IF(AX119="+",BR118+1,0)))</f>
+        <v>0</v>
+      </c>
+      <c r="BS119">
+        <f t="shared" ref="BS119:BS128" si="291">IF(AY119=1,1,IF(AY119="S",BS118,IF(AY119="+",BS118+1,0)))</f>
+        <v>0</v>
+      </c>
+      <c r="BT119">
+        <f t="shared" ref="BT119:BT128" si="292">IF(AZ119=1,1,IF(AZ119="S",BT118,IF(AZ119="+",BT118+1,0)))</f>
+        <v>0</v>
+      </c>
+      <c r="BU119">
+        <f t="shared" ref="BU119:BU128" si="293">IF(BA119=1,1,IF(BA119="S",BU118,IF(BA119="+",BU118+1,0)))</f>
+        <v>0</v>
+      </c>
+      <c r="BV119">
+        <f t="shared" ref="BV119:BV128" si="294">IF(BB119=1,1,IF(BB119="S",BV118,IF(BB119="+",BV118+1,0)))</f>
+        <v>0</v>
+      </c>
+      <c r="BW119">
+        <f t="shared" ref="BW119:BW128" si="295">IF(BC119=1,1,IF(BC119="S",BW118,IF(BC119="+",BW118+1,0)))</f>
+        <v>0</v>
+      </c>
+      <c r="BX119">
+        <f t="shared" ref="BX119:BX128" si="296">IF(BD119=1,1,IF(BD119="S",BX118,IF(BD119="+",BX118+1,0)))</f>
+        <v>0</v>
+      </c>
+      <c r="BY119">
+        <f t="shared" ref="BY119:BY128" si="297">IF(BE119=1,1,IF(BE119="S",BY118,IF(BE119="+",BY118+1,0)))</f>
+        <v>0</v>
+      </c>
+      <c r="BZ119">
+        <f t="shared" ref="BZ119:BZ128" si="298">IF(BF119=1,1,IF(BF119="S",BZ118,IF(BF119="+",BZ118+1,0)))</f>
+        <v>0</v>
+      </c>
+      <c r="CA119">
+        <f t="shared" ref="CA119:CA128" si="299">IF(BG119=1,1,IF(BG119="S",CA118,IF(BG119="+",CA118+1,0)))</f>
+        <v>0</v>
+      </c>
+      <c r="CB119">
+        <f t="shared" ref="CB119:CB128" si="300">IF(BH119=1,1,IF(BH119="S",CB118,IF(BH119="+",CB118+1,0)))</f>
+        <v>0</v>
+      </c>
+      <c r="CC119">
+        <f t="shared" ref="CC119:CC128" si="301">IF(BI119=1,1,IF(BI119="S",CC118,IF(BI119="+",CC118+1,0)))</f>
+        <v>0</v>
+      </c>
+      <c r="CE119" t="str">
+        <f t="shared" ref="CE119:CE128" si="302">TEXT(B119,"000")</f>
+        <v>107</v>
+      </c>
+      <c r="CF119" t="str">
+        <f t="shared" si="181"/>
+        <v>00</v>
+      </c>
+      <c r="CG119" t="str">
+        <f t="shared" si="181"/>
+        <v>00</v>
+      </c>
+      <c r="CH119" t="str">
+        <f t="shared" si="181"/>
+        <v>00</v>
+      </c>
+      <c r="CI119" t="str">
+        <f t="shared" ref="CI119:CI128" si="303">TEXT(BK119,"00")</f>
+        <v>01</v>
+      </c>
+      <c r="CJ119" t="str">
+        <f t="shared" ref="CJ119:CJ128" si="304">TEXT(BL119,"00")</f>
+        <v>07</v>
+      </c>
+      <c r="CK119" t="str">
+        <f t="shared" ref="CK119:CK128" si="305">TEXT(BM119,"00")</f>
+        <v>00</v>
+      </c>
+      <c r="CL119" t="str">
+        <f t="shared" ref="CL119:CL128" si="306">TEXT(BN119,"00")</f>
+        <v>00</v>
+      </c>
+      <c r="CM119" t="str">
+        <f t="shared" ref="CM119:CM128" si="307">TEXT(BO119,"00")</f>
+        <v>00</v>
+      </c>
+      <c r="CN119" t="str">
+        <f t="shared" ref="CN119:CN128" si="308">TEXT(BP119,"00")</f>
+        <v>00</v>
+      </c>
+      <c r="CO119" t="str">
+        <f t="shared" ref="CO119:CO128" si="309">TEXT(BQ119,"00")</f>
+        <v>00</v>
+      </c>
+      <c r="CP119" t="str">
+        <f t="shared" ref="CP119:CP128" si="310">TEXT(BR119,"00")</f>
+        <v>00</v>
+      </c>
+      <c r="CQ119" t="str">
+        <f t="shared" ref="CQ119:CQ128" si="311">TEXT(BS119,"00")</f>
+        <v>00</v>
+      </c>
+      <c r="CR119" t="str">
+        <f t="shared" ref="CR119:CR128" si="312">TEXT(BT119,"00")</f>
+        <v>00</v>
+      </c>
+      <c r="CS119" t="str">
+        <f t="shared" ref="CS119:CS128" si="313">TEXT(BU119,"00")</f>
+        <v>00</v>
+      </c>
+      <c r="CT119" t="str">
+        <f t="shared" ref="CT119:CT128" si="314">TEXT(BV119,"00")</f>
+        <v>00</v>
+      </c>
+      <c r="CU119" t="str">
+        <f t="shared" ref="CU119:CU128" si="315">TEXT(BW119,"00")</f>
+        <v>00</v>
+      </c>
+      <c r="CV119" t="str">
+        <f t="shared" ref="CV119:CV128" si="316">TEXT(BX119,"00")</f>
+        <v>00</v>
+      </c>
+      <c r="CW119" t="str">
+        <f t="shared" ref="CW119:CW128" si="317">TEXT(BY119,"00")</f>
+        <v>00</v>
+      </c>
+      <c r="CX119" t="str">
+        <f t="shared" ref="CX119:CX128" si="318">TEXT(BZ119,"00")</f>
+        <v>00</v>
+      </c>
+      <c r="CY119" t="str">
+        <f t="shared" ref="CY119:CY128" si="319">TEXT(CA119,"00")</f>
+        <v>00</v>
+      </c>
+      <c r="CZ119" t="str">
+        <f t="shared" ref="CZ119:CZ128" si="320">TEXT(CB119,"00")</f>
+        <v>00</v>
+      </c>
+      <c r="DA119" t="str">
+        <f t="shared" ref="DA119:DA128" si="321">TEXT(CC119,"00")</f>
+        <v>00</v>
+      </c>
+      <c r="DB119" t="str">
+        <f t="shared" ref="DB119:DB128" si="322">TEXT(19-COUNTIF(CI119:DA119,"=00"),"00")</f>
+        <v>02</v>
+      </c>
+      <c r="DC119" t="str">
+        <f t="shared" ref="DC119:DC126" si="323">_xlfn.CONCAT(CI119:DB119)</f>
+        <v>0107000000000000000000000000000000000002</v>
+      </c>
+      <c r="DD119" t="str">
+        <f t="shared" ref="DD119:DD126" si="324">_xlfn.CONCAT(C119:U119)</f>
+        <v>Profile</v>
+      </c>
+      <c r="DE119" t="s">
+        <v>242</v>
+      </c>
+      <c r="DF119" t="s">
+        <v>223</v>
+      </c>
+      <c r="DG119" t="s">
+        <v>224</v>
+      </c>
+      <c r="DH119" t="s">
+        <v>225</v>
+      </c>
+      <c r="DI119" t="s">
+        <v>226</v>
+      </c>
+      <c r="DJ119" t="s">
+        <v>227</v>
+      </c>
+      <c r="DK119" t="s">
+        <v>228</v>
+      </c>
+      <c r="DL119" t="str">
+        <f t="shared" ref="DL119:DL126" si="325">_xlfn.TEXTJOIN(",", TRUE,CE119:DK119)</f>
+        <v>107,00,00,00,01,07,00,00,00,00,00,00,00,00,00,00,00,00,00,00,00,00,00,02,0107000000000000000000000000000000000002,Profile,file107,Blk1,Blk2,Blk3,Blk4,Blk5,Blk6</v>
+      </c>
+    </row>
+    <row r="120" spans="2:116" x14ac:dyDescent="0.25">
+      <c r="B120">
+        <f t="shared" si="205"/>
+        <v>108</v>
+      </c>
+      <c r="E120" t="s">
+        <v>234</v>
+      </c>
+      <c r="W120">
+        <f t="shared" si="244"/>
+        <v>0</v>
+      </c>
+      <c r="X120">
+        <f t="shared" si="245"/>
+        <v>0</v>
+      </c>
+      <c r="Y120">
+        <f t="shared" si="246"/>
+        <v>1</v>
+      </c>
+      <c r="Z120">
+        <f t="shared" si="247"/>
+        <v>0</v>
+      </c>
+      <c r="AA120">
+        <f t="shared" si="248"/>
+        <v>0</v>
+      </c>
+      <c r="AB120">
+        <f t="shared" si="249"/>
+        <v>0</v>
+      </c>
+      <c r="AC120">
+        <f t="shared" si="250"/>
+        <v>0</v>
+      </c>
+      <c r="AD120">
+        <f t="shared" si="251"/>
+        <v>0</v>
+      </c>
+      <c r="AE120">
+        <f t="shared" si="252"/>
+        <v>0</v>
+      </c>
+      <c r="AF120">
+        <f t="shared" si="253"/>
+        <v>0</v>
+      </c>
+      <c r="AG120">
+        <f t="shared" si="254"/>
+        <v>0</v>
+      </c>
+      <c r="AH120">
+        <f t="shared" si="255"/>
+        <v>0</v>
+      </c>
+      <c r="AI120">
+        <f t="shared" si="256"/>
+        <v>0</v>
+      </c>
+      <c r="AJ120">
+        <f t="shared" si="257"/>
+        <v>0</v>
+      </c>
+      <c r="AK120">
+        <f t="shared" si="258"/>
+        <v>0</v>
+      </c>
+      <c r="AL120">
+        <f t="shared" si="259"/>
+        <v>0</v>
+      </c>
+      <c r="AM120">
+        <f t="shared" si="260"/>
+        <v>0</v>
+      </c>
+      <c r="AN120">
+        <f t="shared" si="261"/>
+        <v>0</v>
+      </c>
+      <c r="AO120">
+        <f t="shared" si="262"/>
+        <v>0</v>
+      </c>
+      <c r="AP120" s="2" t="str">
+        <f t="shared" si="263"/>
+        <v/>
+      </c>
+      <c r="AQ120" t="str">
+        <f t="shared" si="264"/>
+        <v>S</v>
+      </c>
+      <c r="AR120" t="str">
+        <f t="shared" si="265"/>
+        <v>S</v>
+      </c>
+      <c r="AS120">
+        <f t="shared" si="266"/>
+        <v>1</v>
+      </c>
+      <c r="AT120" t="str">
+        <f t="shared" si="267"/>
+        <v/>
+      </c>
+      <c r="AU120" t="str">
+        <f t="shared" si="268"/>
+        <v/>
+      </c>
+      <c r="AV120" t="str">
+        <f t="shared" si="269"/>
+        <v/>
+      </c>
+      <c r="AW120" t="str">
+        <f t="shared" si="270"/>
+        <v/>
+      </c>
+      <c r="AX120" t="str">
+        <f t="shared" si="271"/>
+        <v/>
+      </c>
+      <c r="AY120" t="str">
+        <f t="shared" si="272"/>
+        <v/>
+      </c>
+      <c r="AZ120" t="str">
+        <f t="shared" si="273"/>
+        <v/>
+      </c>
+      <c r="BA120" t="str">
+        <f t="shared" si="274"/>
+        <v/>
+      </c>
+      <c r="BB120" t="str">
+        <f t="shared" si="275"/>
+        <v/>
+      </c>
+      <c r="BC120" t="str">
+        <f t="shared" si="276"/>
+        <v/>
+      </c>
+      <c r="BD120" t="str">
+        <f t="shared" si="277"/>
+        <v/>
+      </c>
+      <c r="BE120" t="str">
+        <f t="shared" si="278"/>
+        <v/>
+      </c>
+      <c r="BF120" t="str">
+        <f t="shared" si="279"/>
+        <v/>
+      </c>
+      <c r="BG120" t="str">
+        <f t="shared" si="280"/>
+        <v/>
+      </c>
+      <c r="BH120" t="str">
+        <f t="shared" si="281"/>
+        <v/>
+      </c>
+      <c r="BI120" t="str">
+        <f t="shared" si="282"/>
+        <v/>
+      </c>
+      <c r="BK120">
+        <f t="shared" si="283"/>
+        <v>1</v>
+      </c>
+      <c r="BL120">
+        <f t="shared" si="284"/>
+        <v>7</v>
+      </c>
+      <c r="BM120">
+        <f t="shared" si="285"/>
+        <v>1</v>
+      </c>
+      <c r="BN120">
+        <f t="shared" si="286"/>
+        <v>0</v>
+      </c>
+      <c r="BO120">
+        <f t="shared" si="287"/>
+        <v>0</v>
+      </c>
+      <c r="BP120">
+        <f t="shared" si="288"/>
+        <v>0</v>
+      </c>
+      <c r="BQ120">
+        <f t="shared" si="289"/>
+        <v>0</v>
+      </c>
+      <c r="BR120">
+        <f t="shared" si="290"/>
+        <v>0</v>
+      </c>
+      <c r="BS120">
+        <f t="shared" si="291"/>
+        <v>0</v>
+      </c>
+      <c r="BT120">
+        <f t="shared" si="292"/>
+        <v>0</v>
+      </c>
+      <c r="BU120">
+        <f t="shared" si="293"/>
+        <v>0</v>
+      </c>
+      <c r="BV120">
+        <f t="shared" si="294"/>
+        <v>0</v>
+      </c>
+      <c r="BW120">
+        <f t="shared" si="295"/>
+        <v>0</v>
+      </c>
+      <c r="BX120">
+        <f t="shared" si="296"/>
+        <v>0</v>
+      </c>
+      <c r="BY120">
+        <f t="shared" si="297"/>
+        <v>0</v>
+      </c>
+      <c r="BZ120">
+        <f t="shared" si="298"/>
+        <v>0</v>
+      </c>
+      <c r="CA120">
+        <f t="shared" si="299"/>
+        <v>0</v>
+      </c>
+      <c r="CB120">
+        <f t="shared" si="300"/>
+        <v>0</v>
+      </c>
+      <c r="CC120">
+        <f t="shared" si="301"/>
+        <v>0</v>
+      </c>
+      <c r="CE120" t="str">
+        <f t="shared" si="302"/>
+        <v>108</v>
+      </c>
+      <c r="CF120" t="str">
+        <f t="shared" ref="CF120:CH128" si="326">TEXT(0,"00")</f>
+        <v>00</v>
+      </c>
+      <c r="CG120" t="str">
+        <f t="shared" si="326"/>
+        <v>00</v>
+      </c>
+      <c r="CH120" t="str">
+        <f t="shared" si="326"/>
+        <v>00</v>
+      </c>
+      <c r="CI120" t="str">
+        <f t="shared" si="303"/>
+        <v>01</v>
+      </c>
+      <c r="CJ120" t="str">
+        <f t="shared" si="304"/>
+        <v>07</v>
+      </c>
+      <c r="CK120" t="str">
+        <f t="shared" si="305"/>
+        <v>01</v>
+      </c>
+      <c r="CL120" t="str">
+        <f t="shared" si="306"/>
+        <v>00</v>
+      </c>
+      <c r="CM120" t="str">
+        <f t="shared" si="307"/>
+        <v>00</v>
+      </c>
+      <c r="CN120" t="str">
+        <f t="shared" si="308"/>
+        <v>00</v>
+      </c>
+      <c r="CO120" t="str">
+        <f t="shared" si="309"/>
+        <v>00</v>
+      </c>
+      <c r="CP120" t="str">
+        <f t="shared" si="310"/>
+        <v>00</v>
+      </c>
+      <c r="CQ120" t="str">
+        <f t="shared" si="311"/>
+        <v>00</v>
+      </c>
+      <c r="CR120" t="str">
+        <f t="shared" si="312"/>
+        <v>00</v>
+      </c>
+      <c r="CS120" t="str">
+        <f t="shared" si="313"/>
+        <v>00</v>
+      </c>
+      <c r="CT120" t="str">
+        <f t="shared" si="314"/>
+        <v>00</v>
+      </c>
+      <c r="CU120" t="str">
+        <f t="shared" si="315"/>
+        <v>00</v>
+      </c>
+      <c r="CV120" t="str">
+        <f t="shared" si="316"/>
+        <v>00</v>
+      </c>
+      <c r="CW120" t="str">
+        <f t="shared" si="317"/>
+        <v>00</v>
+      </c>
+      <c r="CX120" t="str">
+        <f t="shared" si="318"/>
+        <v>00</v>
+      </c>
+      <c r="CY120" t="str">
+        <f t="shared" si="319"/>
+        <v>00</v>
+      </c>
+      <c r="CZ120" t="str">
+        <f t="shared" si="320"/>
+        <v>00</v>
+      </c>
+      <c r="DA120" t="str">
+        <f t="shared" si="321"/>
+        <v>00</v>
+      </c>
+      <c r="DB120" t="str">
+        <f t="shared" si="322"/>
+        <v>03</v>
+      </c>
+      <c r="DC120" t="str">
+        <f t="shared" si="323"/>
+        <v>0107010000000000000000000000000000000003</v>
+      </c>
+      <c r="DD120" t="str">
+        <f t="shared" si="324"/>
+        <v>Personal</v>
+      </c>
+      <c r="DE120" t="s">
+        <v>251</v>
+      </c>
+      <c r="DF120" t="s">
+        <v>223</v>
+      </c>
+      <c r="DG120" t="s">
+        <v>224</v>
+      </c>
+      <c r="DH120" t="s">
+        <v>225</v>
+      </c>
+      <c r="DI120" t="s">
+        <v>226</v>
+      </c>
+      <c r="DJ120" t="s">
+        <v>227</v>
+      </c>
+      <c r="DK120" t="s">
+        <v>228</v>
+      </c>
+      <c r="DL120" t="str">
+        <f t="shared" si="325"/>
+        <v>108,00,00,00,01,07,01,00,00,00,00,00,00,00,00,00,00,00,00,00,00,00,00,03,0107010000000000000000000000000000000003,Personal,subpages/profile/personal/personal.php,Blk1,Blk2,Blk3,Blk4,Blk5,Blk6</v>
+      </c>
+    </row>
+    <row r="121" spans="2:116" x14ac:dyDescent="0.25">
+      <c r="B121">
+        <f t="shared" si="205"/>
+        <v>109</v>
+      </c>
+      <c r="E121" t="s">
+        <v>235</v>
+      </c>
+      <c r="W121">
+        <f t="shared" si="244"/>
+        <v>0</v>
+      </c>
+      <c r="X121">
+        <f t="shared" si="245"/>
+        <v>0</v>
+      </c>
+      <c r="Y121">
+        <f t="shared" si="246"/>
+        <v>1</v>
+      </c>
+      <c r="Z121">
+        <f t="shared" si="247"/>
+        <v>0</v>
+      </c>
+      <c r="AA121">
+        <f t="shared" si="248"/>
+        <v>0</v>
+      </c>
+      <c r="AB121">
+        <f t="shared" si="249"/>
+        <v>0</v>
+      </c>
+      <c r="AC121">
+        <f t="shared" si="250"/>
+        <v>0</v>
+      </c>
+      <c r="AD121">
+        <f t="shared" si="251"/>
+        <v>0</v>
+      </c>
+      <c r="AE121">
+        <f t="shared" si="252"/>
+        <v>0</v>
+      </c>
+      <c r="AF121">
+        <f t="shared" si="253"/>
+        <v>0</v>
+      </c>
+      <c r="AG121">
+        <f t="shared" si="254"/>
+        <v>0</v>
+      </c>
+      <c r="AH121">
+        <f t="shared" si="255"/>
+        <v>0</v>
+      </c>
+      <c r="AI121">
+        <f t="shared" si="256"/>
+        <v>0</v>
+      </c>
+      <c r="AJ121">
+        <f t="shared" si="257"/>
+        <v>0</v>
+      </c>
+      <c r="AK121">
+        <f t="shared" si="258"/>
+        <v>0</v>
+      </c>
+      <c r="AL121">
+        <f t="shared" si="259"/>
+        <v>0</v>
+      </c>
+      <c r="AM121">
+        <f t="shared" si="260"/>
+        <v>0</v>
+      </c>
+      <c r="AN121">
+        <f t="shared" si="261"/>
+        <v>0</v>
+      </c>
+      <c r="AO121">
+        <f t="shared" si="262"/>
+        <v>0</v>
+      </c>
+      <c r="AP121" s="2" t="str">
+        <f t="shared" si="263"/>
+        <v/>
+      </c>
+      <c r="AQ121" t="str">
+        <f t="shared" si="264"/>
+        <v>S</v>
+      </c>
+      <c r="AR121" t="str">
+        <f t="shared" si="265"/>
+        <v>S</v>
+      </c>
+      <c r="AS121" t="str">
+        <f t="shared" si="266"/>
+        <v>+</v>
+      </c>
+      <c r="AT121" t="str">
+        <f t="shared" si="267"/>
+        <v/>
+      </c>
+      <c r="AU121" t="str">
+        <f t="shared" si="268"/>
+        <v/>
+      </c>
+      <c r="AV121" t="str">
+        <f t="shared" si="269"/>
+        <v/>
+      </c>
+      <c r="AW121" t="str">
+        <f t="shared" si="270"/>
+        <v/>
+      </c>
+      <c r="AX121" t="str">
+        <f t="shared" si="271"/>
+        <v/>
+      </c>
+      <c r="AY121" t="str">
+        <f t="shared" si="272"/>
+        <v/>
+      </c>
+      <c r="AZ121" t="str">
+        <f t="shared" si="273"/>
+        <v/>
+      </c>
+      <c r="BA121" t="str">
+        <f t="shared" si="274"/>
+        <v/>
+      </c>
+      <c r="BB121" t="str">
+        <f t="shared" si="275"/>
+        <v/>
+      </c>
+      <c r="BC121" t="str">
+        <f t="shared" si="276"/>
+        <v/>
+      </c>
+      <c r="BD121" t="str">
+        <f t="shared" si="277"/>
+        <v/>
+      </c>
+      <c r="BE121" t="str">
+        <f t="shared" si="278"/>
+        <v/>
+      </c>
+      <c r="BF121" t="str">
+        <f t="shared" si="279"/>
+        <v/>
+      </c>
+      <c r="BG121" t="str">
+        <f t="shared" si="280"/>
+        <v/>
+      </c>
+      <c r="BH121" t="str">
+        <f t="shared" si="281"/>
+        <v/>
+      </c>
+      <c r="BI121" t="str">
+        <f t="shared" si="282"/>
+        <v/>
+      </c>
+      <c r="BK121">
+        <f t="shared" si="283"/>
+        <v>1</v>
+      </c>
+      <c r="BL121">
+        <f t="shared" si="284"/>
+        <v>7</v>
+      </c>
+      <c r="BM121">
+        <f t="shared" si="285"/>
+        <v>2</v>
+      </c>
+      <c r="BN121">
+        <f t="shared" si="286"/>
+        <v>0</v>
+      </c>
+      <c r="BO121">
+        <f t="shared" si="287"/>
+        <v>0</v>
+      </c>
+      <c r="BP121">
+        <f t="shared" si="288"/>
+        <v>0</v>
+      </c>
+      <c r="BQ121">
+        <f t="shared" si="289"/>
+        <v>0</v>
+      </c>
+      <c r="BR121">
+        <f t="shared" si="290"/>
+        <v>0</v>
+      </c>
+      <c r="BS121">
+        <f t="shared" si="291"/>
+        <v>0</v>
+      </c>
+      <c r="BT121">
+        <f t="shared" si="292"/>
+        <v>0</v>
+      </c>
+      <c r="BU121">
+        <f t="shared" si="293"/>
+        <v>0</v>
+      </c>
+      <c r="BV121">
+        <f t="shared" si="294"/>
+        <v>0</v>
+      </c>
+      <c r="BW121">
+        <f t="shared" si="295"/>
+        <v>0</v>
+      </c>
+      <c r="BX121">
+        <f t="shared" si="296"/>
+        <v>0</v>
+      </c>
+      <c r="BY121">
+        <f t="shared" si="297"/>
+        <v>0</v>
+      </c>
+      <c r="BZ121">
+        <f t="shared" si="298"/>
+        <v>0</v>
+      </c>
+      <c r="CA121">
+        <f t="shared" si="299"/>
+        <v>0</v>
+      </c>
+      <c r="CB121">
+        <f t="shared" si="300"/>
+        <v>0</v>
+      </c>
+      <c r="CC121">
+        <f t="shared" si="301"/>
+        <v>0</v>
+      </c>
+      <c r="CE121" t="str">
+        <f t="shared" si="302"/>
+        <v>109</v>
+      </c>
+      <c r="CF121" t="str">
+        <f t="shared" si="326"/>
+        <v>00</v>
+      </c>
+      <c r="CG121" t="str">
+        <f t="shared" si="326"/>
+        <v>00</v>
+      </c>
+      <c r="CH121" t="str">
+        <f t="shared" si="326"/>
+        <v>00</v>
+      </c>
+      <c r="CI121" t="str">
+        <f t="shared" si="303"/>
+        <v>01</v>
+      </c>
+      <c r="CJ121" t="str">
+        <f t="shared" si="304"/>
+        <v>07</v>
+      </c>
+      <c r="CK121" t="str">
+        <f t="shared" si="305"/>
+        <v>02</v>
+      </c>
+      <c r="CL121" t="str">
+        <f t="shared" si="306"/>
+        <v>00</v>
+      </c>
+      <c r="CM121" t="str">
+        <f t="shared" si="307"/>
+        <v>00</v>
+      </c>
+      <c r="CN121" t="str">
+        <f t="shared" si="308"/>
+        <v>00</v>
+      </c>
+      <c r="CO121" t="str">
+        <f t="shared" si="309"/>
+        <v>00</v>
+      </c>
+      <c r="CP121" t="str">
+        <f t="shared" si="310"/>
+        <v>00</v>
+      </c>
+      <c r="CQ121" t="str">
+        <f t="shared" si="311"/>
+        <v>00</v>
+      </c>
+      <c r="CR121" t="str">
+        <f t="shared" si="312"/>
+        <v>00</v>
+      </c>
+      <c r="CS121" t="str">
+        <f t="shared" si="313"/>
+        <v>00</v>
+      </c>
+      <c r="CT121" t="str">
+        <f t="shared" si="314"/>
+        <v>00</v>
+      </c>
+      <c r="CU121" t="str">
+        <f t="shared" si="315"/>
+        <v>00</v>
+      </c>
+      <c r="CV121" t="str">
+        <f t="shared" si="316"/>
+        <v>00</v>
+      </c>
+      <c r="CW121" t="str">
+        <f t="shared" si="317"/>
+        <v>00</v>
+      </c>
+      <c r="CX121" t="str">
+        <f t="shared" si="318"/>
+        <v>00</v>
+      </c>
+      <c r="CY121" t="str">
+        <f t="shared" si="319"/>
+        <v>00</v>
+      </c>
+      <c r="CZ121" t="str">
+        <f t="shared" si="320"/>
+        <v>00</v>
+      </c>
+      <c r="DA121" t="str">
+        <f t="shared" si="321"/>
+        <v>00</v>
+      </c>
+      <c r="DB121" t="str">
+        <f t="shared" si="322"/>
+        <v>03</v>
+      </c>
+      <c r="DC121" t="str">
+        <f t="shared" si="323"/>
+        <v>0107020000000000000000000000000000000003</v>
+      </c>
+      <c r="DD121" t="str">
+        <f t="shared" si="324"/>
+        <v>Account &amp; Security</v>
+      </c>
+      <c r="DE121" t="s">
+        <v>243</v>
+      </c>
+      <c r="DF121" t="s">
+        <v>223</v>
+      </c>
+      <c r="DG121" t="s">
+        <v>224</v>
+      </c>
+      <c r="DH121" t="s">
+        <v>225</v>
+      </c>
+      <c r="DI121" t="s">
+        <v>226</v>
+      </c>
+      <c r="DJ121" t="s">
+        <v>227</v>
+      </c>
+      <c r="DK121" t="s">
+        <v>228</v>
+      </c>
+      <c r="DL121" t="str">
+        <f t="shared" si="325"/>
+        <v>109,00,00,00,01,07,02,00,00,00,00,00,00,00,00,00,00,00,00,00,00,00,00,03,0107020000000000000000000000000000000003,Account &amp; Security,file109,Blk1,Blk2,Blk3,Blk4,Blk5,Blk6</v>
+      </c>
+    </row>
+    <row r="122" spans="2:116" x14ac:dyDescent="0.25">
+      <c r="B122">
+        <f t="shared" si="205"/>
+        <v>110</v>
+      </c>
+      <c r="F122" t="s">
+        <v>238</v>
+      </c>
+      <c r="W122">
+        <f t="shared" si="244"/>
+        <v>0</v>
+      </c>
+      <c r="X122">
+        <f t="shared" si="245"/>
+        <v>0</v>
+      </c>
+      <c r="Y122">
+        <f t="shared" si="246"/>
+        <v>0</v>
+      </c>
+      <c r="Z122">
+        <f t="shared" si="247"/>
+        <v>1</v>
+      </c>
+      <c r="AA122">
+        <f t="shared" si="248"/>
+        <v>0</v>
+      </c>
+      <c r="AB122">
+        <f t="shared" si="249"/>
+        <v>0</v>
+      </c>
+      <c r="AC122">
+        <f t="shared" si="250"/>
+        <v>0</v>
+      </c>
+      <c r="AD122">
+        <f t="shared" si="251"/>
+        <v>0</v>
+      </c>
+      <c r="AE122">
+        <f t="shared" si="252"/>
+        <v>0</v>
+      </c>
+      <c r="AF122">
+        <f t="shared" si="253"/>
+        <v>0</v>
+      </c>
+      <c r="AG122">
+        <f t="shared" si="254"/>
+        <v>0</v>
+      </c>
+      <c r="AH122">
+        <f t="shared" si="255"/>
+        <v>0</v>
+      </c>
+      <c r="AI122">
+        <f t="shared" si="256"/>
+        <v>0</v>
+      </c>
+      <c r="AJ122">
+        <f t="shared" si="257"/>
+        <v>0</v>
+      </c>
+      <c r="AK122">
+        <f t="shared" si="258"/>
+        <v>0</v>
+      </c>
+      <c r="AL122">
+        <f t="shared" si="259"/>
+        <v>0</v>
+      </c>
+      <c r="AM122">
+        <f t="shared" si="260"/>
+        <v>0</v>
+      </c>
+      <c r="AN122">
+        <f t="shared" si="261"/>
+        <v>0</v>
+      </c>
+      <c r="AO122">
+        <f t="shared" si="262"/>
+        <v>0</v>
+      </c>
+      <c r="AP122" s="2" t="str">
+        <f t="shared" si="263"/>
+        <v/>
+      </c>
+      <c r="AQ122" t="str">
+        <f t="shared" si="264"/>
+        <v>S</v>
+      </c>
+      <c r="AR122" t="str">
+        <f t="shared" si="265"/>
+        <v>S</v>
+      </c>
+      <c r="AS122" t="str">
+        <f t="shared" si="266"/>
+        <v>S</v>
+      </c>
+      <c r="AT122">
+        <f t="shared" si="267"/>
+        <v>1</v>
+      </c>
+      <c r="AU122" t="str">
+        <f t="shared" si="268"/>
+        <v/>
+      </c>
+      <c r="AV122" t="str">
+        <f t="shared" si="269"/>
+        <v/>
+      </c>
+      <c r="AW122" t="str">
+        <f t="shared" si="270"/>
+        <v/>
+      </c>
+      <c r="AX122" t="str">
+        <f t="shared" si="271"/>
+        <v/>
+      </c>
+      <c r="AY122" t="str">
+        <f t="shared" si="272"/>
+        <v/>
+      </c>
+      <c r="AZ122" t="str">
+        <f t="shared" si="273"/>
+        <v/>
+      </c>
+      <c r="BA122" t="str">
+        <f t="shared" si="274"/>
+        <v/>
+      </c>
+      <c r="BB122" t="str">
+        <f t="shared" si="275"/>
+        <v/>
+      </c>
+      <c r="BC122" t="str">
+        <f t="shared" si="276"/>
+        <v/>
+      </c>
+      <c r="BD122" t="str">
+        <f t="shared" si="277"/>
+        <v/>
+      </c>
+      <c r="BE122" t="str">
+        <f t="shared" si="278"/>
+        <v/>
+      </c>
+      <c r="BF122" t="str">
+        <f t="shared" si="279"/>
+        <v/>
+      </c>
+      <c r="BG122" t="str">
+        <f t="shared" si="280"/>
+        <v/>
+      </c>
+      <c r="BH122" t="str">
+        <f t="shared" si="281"/>
+        <v/>
+      </c>
+      <c r="BI122" t="str">
+        <f t="shared" si="282"/>
+        <v/>
+      </c>
+      <c r="BK122">
+        <f t="shared" si="283"/>
+        <v>1</v>
+      </c>
+      <c r="BL122">
+        <f t="shared" si="284"/>
+        <v>7</v>
+      </c>
+      <c r="BM122">
+        <f t="shared" si="285"/>
+        <v>2</v>
+      </c>
+      <c r="BN122">
+        <f t="shared" si="286"/>
+        <v>1</v>
+      </c>
+      <c r="BO122">
+        <f t="shared" si="287"/>
+        <v>0</v>
+      </c>
+      <c r="BP122">
+        <f t="shared" si="288"/>
+        <v>0</v>
+      </c>
+      <c r="BQ122">
+        <f t="shared" si="289"/>
+        <v>0</v>
+      </c>
+      <c r="BR122">
+        <f t="shared" si="290"/>
+        <v>0</v>
+      </c>
+      <c r="BS122">
+        <f t="shared" si="291"/>
+        <v>0</v>
+      </c>
+      <c r="BT122">
+        <f t="shared" si="292"/>
+        <v>0</v>
+      </c>
+      <c r="BU122">
+        <f t="shared" si="293"/>
+        <v>0</v>
+      </c>
+      <c r="BV122">
+        <f t="shared" si="294"/>
+        <v>0</v>
+      </c>
+      <c r="BW122">
+        <f t="shared" si="295"/>
+        <v>0</v>
+      </c>
+      <c r="BX122">
+        <f t="shared" si="296"/>
+        <v>0</v>
+      </c>
+      <c r="BY122">
+        <f t="shared" si="297"/>
+        <v>0</v>
+      </c>
+      <c r="BZ122">
+        <f t="shared" si="298"/>
+        <v>0</v>
+      </c>
+      <c r="CA122">
+        <f t="shared" si="299"/>
+        <v>0</v>
+      </c>
+      <c r="CB122">
+        <f t="shared" si="300"/>
+        <v>0</v>
+      </c>
+      <c r="CC122">
+        <f t="shared" si="301"/>
+        <v>0</v>
+      </c>
+      <c r="CE122" t="str">
+        <f t="shared" si="302"/>
+        <v>110</v>
+      </c>
+      <c r="CF122" t="str">
+        <f t="shared" si="326"/>
+        <v>00</v>
+      </c>
+      <c r="CG122" t="str">
+        <f t="shared" si="326"/>
+        <v>00</v>
+      </c>
+      <c r="CH122" t="str">
+        <f t="shared" si="326"/>
+        <v>00</v>
+      </c>
+      <c r="CI122" t="str">
+        <f t="shared" si="303"/>
+        <v>01</v>
+      </c>
+      <c r="CJ122" t="str">
+        <f t="shared" si="304"/>
+        <v>07</v>
+      </c>
+      <c r="CK122" t="str">
+        <f t="shared" si="305"/>
+        <v>02</v>
+      </c>
+      <c r="CL122" t="str">
+        <f t="shared" si="306"/>
+        <v>01</v>
+      </c>
+      <c r="CM122" t="str">
+        <f t="shared" si="307"/>
+        <v>00</v>
+      </c>
+      <c r="CN122" t="str">
+        <f t="shared" si="308"/>
+        <v>00</v>
+      </c>
+      <c r="CO122" t="str">
+        <f t="shared" si="309"/>
+        <v>00</v>
+      </c>
+      <c r="CP122" t="str">
+        <f t="shared" si="310"/>
+        <v>00</v>
+      </c>
+      <c r="CQ122" t="str">
+        <f t="shared" si="311"/>
+        <v>00</v>
+      </c>
+      <c r="CR122" t="str">
+        <f t="shared" si="312"/>
+        <v>00</v>
+      </c>
+      <c r="CS122" t="str">
+        <f t="shared" si="313"/>
+        <v>00</v>
+      </c>
+      <c r="CT122" t="str">
+        <f t="shared" si="314"/>
+        <v>00</v>
+      </c>
+      <c r="CU122" t="str">
+        <f t="shared" si="315"/>
+        <v>00</v>
+      </c>
+      <c r="CV122" t="str">
+        <f t="shared" si="316"/>
+        <v>00</v>
+      </c>
+      <c r="CW122" t="str">
+        <f t="shared" si="317"/>
+        <v>00</v>
+      </c>
+      <c r="CX122" t="str">
+        <f t="shared" si="318"/>
+        <v>00</v>
+      </c>
+      <c r="CY122" t="str">
+        <f t="shared" si="319"/>
+        <v>00</v>
+      </c>
+      <c r="CZ122" t="str">
+        <f t="shared" si="320"/>
+        <v>00</v>
+      </c>
+      <c r="DA122" t="str">
+        <f t="shared" si="321"/>
+        <v>00</v>
+      </c>
+      <c r="DB122" t="str">
+        <f t="shared" si="322"/>
+        <v>04</v>
+      </c>
+      <c r="DC122" t="str">
+        <f t="shared" si="323"/>
+        <v>0107020100000000000000000000000000000004</v>
+      </c>
+      <c r="DD122" t="str">
+        <f t="shared" si="324"/>
+        <v>Password</v>
+      </c>
+      <c r="DE122" t="s">
+        <v>244</v>
+      </c>
+      <c r="DF122" t="s">
+        <v>223</v>
+      </c>
+      <c r="DG122" t="s">
+        <v>224</v>
+      </c>
+      <c r="DH122" t="s">
+        <v>225</v>
+      </c>
+      <c r="DI122" t="s">
+        <v>226</v>
+      </c>
+      <c r="DJ122" t="s">
+        <v>227</v>
+      </c>
+      <c r="DK122" t="s">
+        <v>228</v>
+      </c>
+      <c r="DL122" t="str">
+        <f t="shared" si="325"/>
+        <v>110,00,00,00,01,07,02,01,00,00,00,00,00,00,00,00,00,00,00,00,00,00,00,04,0107020100000000000000000000000000000004,Password,file110,Blk1,Blk2,Blk3,Blk4,Blk5,Blk6</v>
+      </c>
+    </row>
+    <row r="123" spans="2:116" x14ac:dyDescent="0.25">
+      <c r="B123">
+        <f t="shared" si="205"/>
+        <v>111</v>
+      </c>
+      <c r="F123" t="s">
+        <v>239</v>
+      </c>
+      <c r="W123">
+        <f t="shared" si="244"/>
+        <v>0</v>
+      </c>
+      <c r="X123">
+        <f t="shared" si="245"/>
+        <v>0</v>
+      </c>
+      <c r="Y123">
+        <f t="shared" si="246"/>
+        <v>0</v>
+      </c>
+      <c r="Z123">
+        <f t="shared" si="247"/>
+        <v>1</v>
+      </c>
+      <c r="AA123">
+        <f t="shared" si="248"/>
+        <v>0</v>
+      </c>
+      <c r="AB123">
+        <f t="shared" si="249"/>
+        <v>0</v>
+      </c>
+      <c r="AC123">
+        <f t="shared" si="250"/>
+        <v>0</v>
+      </c>
+      <c r="AD123">
+        <f t="shared" si="251"/>
+        <v>0</v>
+      </c>
+      <c r="AE123">
+        <f t="shared" si="252"/>
+        <v>0</v>
+      </c>
+      <c r="AF123">
+        <f t="shared" si="253"/>
+        <v>0</v>
+      </c>
+      <c r="AG123">
+        <f t="shared" si="254"/>
+        <v>0</v>
+      </c>
+      <c r="AH123">
+        <f t="shared" si="255"/>
+        <v>0</v>
+      </c>
+      <c r="AI123">
+        <f t="shared" si="256"/>
+        <v>0</v>
+      </c>
+      <c r="AJ123">
+        <f t="shared" si="257"/>
+        <v>0</v>
+      </c>
+      <c r="AK123">
+        <f t="shared" si="258"/>
+        <v>0</v>
+      </c>
+      <c r="AL123">
+        <f t="shared" si="259"/>
+        <v>0</v>
+      </c>
+      <c r="AM123">
+        <f t="shared" si="260"/>
+        <v>0</v>
+      </c>
+      <c r="AN123">
+        <f t="shared" si="261"/>
+        <v>0</v>
+      </c>
+      <c r="AO123">
+        <f t="shared" si="262"/>
+        <v>0</v>
+      </c>
+      <c r="AP123" s="2" t="str">
+        <f t="shared" si="263"/>
+        <v/>
+      </c>
+      <c r="AQ123" t="str">
+        <f t="shared" si="264"/>
+        <v>S</v>
+      </c>
+      <c r="AR123" t="str">
+        <f t="shared" si="265"/>
+        <v>S</v>
+      </c>
+      <c r="AS123" t="str">
+        <f t="shared" si="266"/>
+        <v>S</v>
+      </c>
+      <c r="AT123" t="str">
+        <f t="shared" si="267"/>
+        <v>+</v>
+      </c>
+      <c r="AU123" t="str">
+        <f t="shared" si="268"/>
+        <v/>
+      </c>
+      <c r="AV123" t="str">
+        <f t="shared" si="269"/>
+        <v/>
+      </c>
+      <c r="AW123" t="str">
+        <f t="shared" si="270"/>
+        <v/>
+      </c>
+      <c r="AX123" t="str">
+        <f t="shared" si="271"/>
+        <v/>
+      </c>
+      <c r="AY123" t="str">
+        <f t="shared" si="272"/>
+        <v/>
+      </c>
+      <c r="AZ123" t="str">
+        <f t="shared" si="273"/>
+        <v/>
+      </c>
+      <c r="BA123" t="str">
+        <f t="shared" si="274"/>
+        <v/>
+      </c>
+      <c r="BB123" t="str">
+        <f t="shared" si="275"/>
+        <v/>
+      </c>
+      <c r="BC123" t="str">
+        <f t="shared" si="276"/>
+        <v/>
+      </c>
+      <c r="BD123" t="str">
+        <f t="shared" si="277"/>
+        <v/>
+      </c>
+      <c r="BE123" t="str">
+        <f t="shared" si="278"/>
+        <v/>
+      </c>
+      <c r="BF123" t="str">
+        <f t="shared" si="279"/>
+        <v/>
+      </c>
+      <c r="BG123" t="str">
+        <f t="shared" si="280"/>
+        <v/>
+      </c>
+      <c r="BH123" t="str">
+        <f t="shared" si="281"/>
+        <v/>
+      </c>
+      <c r="BI123" t="str">
+        <f t="shared" si="282"/>
+        <v/>
+      </c>
+      <c r="BK123">
+        <f t="shared" si="283"/>
+        <v>1</v>
+      </c>
+      <c r="BL123">
+        <f t="shared" si="284"/>
+        <v>7</v>
+      </c>
+      <c r="BM123">
+        <f t="shared" si="285"/>
+        <v>2</v>
+      </c>
+      <c r="BN123">
+        <f t="shared" si="286"/>
+        <v>2</v>
+      </c>
+      <c r="BO123">
+        <f t="shared" si="287"/>
+        <v>0</v>
+      </c>
+      <c r="BP123">
+        <f t="shared" si="288"/>
+        <v>0</v>
+      </c>
+      <c r="BQ123">
+        <f t="shared" si="289"/>
+        <v>0</v>
+      </c>
+      <c r="BR123">
+        <f t="shared" si="290"/>
+        <v>0</v>
+      </c>
+      <c r="BS123">
+        <f t="shared" si="291"/>
+        <v>0</v>
+      </c>
+      <c r="BT123">
+        <f t="shared" si="292"/>
+        <v>0</v>
+      </c>
+      <c r="BU123">
+        <f t="shared" si="293"/>
+        <v>0</v>
+      </c>
+      <c r="BV123">
+        <f t="shared" si="294"/>
+        <v>0</v>
+      </c>
+      <c r="BW123">
+        <f t="shared" si="295"/>
+        <v>0</v>
+      </c>
+      <c r="BX123">
+        <f t="shared" si="296"/>
+        <v>0</v>
+      </c>
+      <c r="BY123">
+        <f t="shared" si="297"/>
+        <v>0</v>
+      </c>
+      <c r="BZ123">
+        <f t="shared" si="298"/>
+        <v>0</v>
+      </c>
+      <c r="CA123">
+        <f t="shared" si="299"/>
+        <v>0</v>
+      </c>
+      <c r="CB123">
+        <f t="shared" si="300"/>
+        <v>0</v>
+      </c>
+      <c r="CC123">
+        <f t="shared" si="301"/>
+        <v>0</v>
+      </c>
+      <c r="CE123" t="str">
+        <f t="shared" si="302"/>
+        <v>111</v>
+      </c>
+      <c r="CF123" t="str">
+        <f t="shared" si="326"/>
+        <v>00</v>
+      </c>
+      <c r="CG123" t="str">
+        <f t="shared" si="326"/>
+        <v>00</v>
+      </c>
+      <c r="CH123" t="str">
+        <f t="shared" si="326"/>
+        <v>00</v>
+      </c>
+      <c r="CI123" t="str">
+        <f t="shared" si="303"/>
+        <v>01</v>
+      </c>
+      <c r="CJ123" t="str">
+        <f t="shared" si="304"/>
+        <v>07</v>
+      </c>
+      <c r="CK123" t="str">
+        <f t="shared" si="305"/>
+        <v>02</v>
+      </c>
+      <c r="CL123" t="str">
+        <f t="shared" si="306"/>
+        <v>02</v>
+      </c>
+      <c r="CM123" t="str">
+        <f t="shared" si="307"/>
+        <v>00</v>
+      </c>
+      <c r="CN123" t="str">
+        <f t="shared" si="308"/>
+        <v>00</v>
+      </c>
+      <c r="CO123" t="str">
+        <f t="shared" si="309"/>
+        <v>00</v>
+      </c>
+      <c r="CP123" t="str">
+        <f t="shared" si="310"/>
+        <v>00</v>
+      </c>
+      <c r="CQ123" t="str">
+        <f t="shared" si="311"/>
+        <v>00</v>
+      </c>
+      <c r="CR123" t="str">
+        <f t="shared" si="312"/>
+        <v>00</v>
+      </c>
+      <c r="CS123" t="str">
+        <f t="shared" si="313"/>
+        <v>00</v>
+      </c>
+      <c r="CT123" t="str">
+        <f t="shared" si="314"/>
+        <v>00</v>
+      </c>
+      <c r="CU123" t="str">
+        <f t="shared" si="315"/>
+        <v>00</v>
+      </c>
+      <c r="CV123" t="str">
+        <f t="shared" si="316"/>
+        <v>00</v>
+      </c>
+      <c r="CW123" t="str">
+        <f t="shared" si="317"/>
+        <v>00</v>
+      </c>
+      <c r="CX123" t="str">
+        <f t="shared" si="318"/>
+        <v>00</v>
+      </c>
+      <c r="CY123" t="str">
+        <f t="shared" si="319"/>
+        <v>00</v>
+      </c>
+      <c r="CZ123" t="str">
+        <f t="shared" si="320"/>
+        <v>00</v>
+      </c>
+      <c r="DA123" t="str">
+        <f t="shared" si="321"/>
+        <v>00</v>
+      </c>
+      <c r="DB123" t="str">
+        <f t="shared" si="322"/>
+        <v>04</v>
+      </c>
+      <c r="DC123" t="str">
+        <f t="shared" si="323"/>
+        <v>0107020200000000000000000000000000000004</v>
+      </c>
+      <c r="DD123" t="str">
+        <f t="shared" si="324"/>
+        <v>Two-Factor Authentication</v>
+      </c>
+      <c r="DE123" t="s">
+        <v>245</v>
+      </c>
+      <c r="DF123" t="s">
+        <v>223</v>
+      </c>
+      <c r="DG123" t="s">
+        <v>224</v>
+      </c>
+      <c r="DH123" t="s">
+        <v>225</v>
+      </c>
+      <c r="DI123" t="s">
+        <v>226</v>
+      </c>
+      <c r="DJ123" t="s">
+        <v>227</v>
+      </c>
+      <c r="DK123" t="s">
+        <v>228</v>
+      </c>
+      <c r="DL123" t="str">
+        <f t="shared" si="325"/>
+        <v>111,00,00,00,01,07,02,02,00,00,00,00,00,00,00,00,00,00,00,00,00,00,00,04,0107020200000000000000000000000000000004,Two-Factor Authentication,file111,Blk1,Blk2,Blk3,Blk4,Blk5,Blk6</v>
+      </c>
+    </row>
+    <row r="124" spans="2:116" x14ac:dyDescent="0.25">
+      <c r="B124">
+        <f t="shared" si="205"/>
+        <v>112</v>
+      </c>
+      <c r="F124" t="s">
+        <v>240</v>
+      </c>
+      <c r="W124">
+        <f t="shared" si="244"/>
+        <v>0</v>
+      </c>
+      <c r="X124">
+        <f t="shared" si="245"/>
+        <v>0</v>
+      </c>
+      <c r="Y124">
+        <f t="shared" si="246"/>
+        <v>0</v>
+      </c>
+      <c r="Z124">
+        <f t="shared" si="247"/>
+        <v>1</v>
+      </c>
+      <c r="AA124">
+        <f t="shared" si="248"/>
+        <v>0</v>
+      </c>
+      <c r="AB124">
+        <f t="shared" si="249"/>
+        <v>0</v>
+      </c>
+      <c r="AC124">
+        <f t="shared" si="250"/>
+        <v>0</v>
+      </c>
+      <c r="AD124">
+        <f t="shared" si="251"/>
+        <v>0</v>
+      </c>
+      <c r="AE124">
+        <f t="shared" si="252"/>
+        <v>0</v>
+      </c>
+      <c r="AF124">
+        <f t="shared" si="253"/>
+        <v>0</v>
+      </c>
+      <c r="AG124">
+        <f t="shared" si="254"/>
+        <v>0</v>
+      </c>
+      <c r="AH124">
+        <f t="shared" si="255"/>
+        <v>0</v>
+      </c>
+      <c r="AI124">
+        <f t="shared" si="256"/>
+        <v>0</v>
+      </c>
+      <c r="AJ124">
+        <f t="shared" si="257"/>
+        <v>0</v>
+      </c>
+      <c r="AK124">
+        <f t="shared" si="258"/>
+        <v>0</v>
+      </c>
+      <c r="AL124">
+        <f t="shared" si="259"/>
+        <v>0</v>
+      </c>
+      <c r="AM124">
+        <f t="shared" si="260"/>
+        <v>0</v>
+      </c>
+      <c r="AN124">
+        <f t="shared" si="261"/>
+        <v>0</v>
+      </c>
+      <c r="AO124">
+        <f t="shared" si="262"/>
+        <v>0</v>
+      </c>
+      <c r="AP124" s="2" t="str">
+        <f t="shared" si="263"/>
+        <v/>
+      </c>
+      <c r="AQ124" t="str">
+        <f t="shared" si="264"/>
+        <v>S</v>
+      </c>
+      <c r="AR124" t="str">
+        <f t="shared" si="265"/>
+        <v>S</v>
+      </c>
+      <c r="AS124" t="str">
+        <f t="shared" si="266"/>
+        <v>S</v>
+      </c>
+      <c r="AT124" t="str">
+        <f t="shared" si="267"/>
+        <v>+</v>
+      </c>
+      <c r="AU124" t="str">
+        <f t="shared" si="268"/>
+        <v/>
+      </c>
+      <c r="AV124" t="str">
+        <f t="shared" si="269"/>
+        <v/>
+      </c>
+      <c r="AW124" t="str">
+        <f t="shared" si="270"/>
+        <v/>
+      </c>
+      <c r="AX124" t="str">
+        <f t="shared" si="271"/>
+        <v/>
+      </c>
+      <c r="AY124" t="str">
+        <f t="shared" si="272"/>
+        <v/>
+      </c>
+      <c r="AZ124" t="str">
+        <f t="shared" si="273"/>
+        <v/>
+      </c>
+      <c r="BA124" t="str">
+        <f t="shared" si="274"/>
+        <v/>
+      </c>
+      <c r="BB124" t="str">
+        <f t="shared" si="275"/>
+        <v/>
+      </c>
+      <c r="BC124" t="str">
+        <f t="shared" si="276"/>
+        <v/>
+      </c>
+      <c r="BD124" t="str">
+        <f t="shared" si="277"/>
+        <v/>
+      </c>
+      <c r="BE124" t="str">
+        <f t="shared" si="278"/>
+        <v/>
+      </c>
+      <c r="BF124" t="str">
+        <f t="shared" si="279"/>
+        <v/>
+      </c>
+      <c r="BG124" t="str">
+        <f t="shared" si="280"/>
+        <v/>
+      </c>
+      <c r="BH124" t="str">
+        <f t="shared" si="281"/>
+        <v/>
+      </c>
+      <c r="BI124" t="str">
+        <f t="shared" si="282"/>
+        <v/>
+      </c>
+      <c r="BK124">
+        <f t="shared" si="283"/>
+        <v>1</v>
+      </c>
+      <c r="BL124">
+        <f t="shared" si="284"/>
+        <v>7</v>
+      </c>
+      <c r="BM124">
+        <f t="shared" si="285"/>
+        <v>2</v>
+      </c>
+      <c r="BN124">
+        <f t="shared" si="286"/>
+        <v>3</v>
+      </c>
+      <c r="BO124">
+        <f t="shared" si="287"/>
+        <v>0</v>
+      </c>
+      <c r="BP124">
+        <f t="shared" si="288"/>
+        <v>0</v>
+      </c>
+      <c r="BQ124">
+        <f t="shared" si="289"/>
+        <v>0</v>
+      </c>
+      <c r="BR124">
+        <f t="shared" si="290"/>
+        <v>0</v>
+      </c>
+      <c r="BS124">
+        <f t="shared" si="291"/>
+        <v>0</v>
+      </c>
+      <c r="BT124">
+        <f t="shared" si="292"/>
+        <v>0</v>
+      </c>
+      <c r="BU124">
+        <f t="shared" si="293"/>
+        <v>0</v>
+      </c>
+      <c r="BV124">
+        <f t="shared" si="294"/>
+        <v>0</v>
+      </c>
+      <c r="BW124">
+        <f t="shared" si="295"/>
+        <v>0</v>
+      </c>
+      <c r="BX124">
+        <f t="shared" si="296"/>
+        <v>0</v>
+      </c>
+      <c r="BY124">
+        <f t="shared" si="297"/>
+        <v>0</v>
+      </c>
+      <c r="BZ124">
+        <f t="shared" si="298"/>
+        <v>0</v>
+      </c>
+      <c r="CA124">
+        <f t="shared" si="299"/>
+        <v>0</v>
+      </c>
+      <c r="CB124">
+        <f t="shared" si="300"/>
+        <v>0</v>
+      </c>
+      <c r="CC124">
+        <f t="shared" si="301"/>
+        <v>0</v>
+      </c>
+      <c r="CE124" t="str">
+        <f t="shared" si="302"/>
+        <v>112</v>
+      </c>
+      <c r="CF124" t="str">
+        <f t="shared" si="326"/>
+        <v>00</v>
+      </c>
+      <c r="CG124" t="str">
+        <f t="shared" si="326"/>
+        <v>00</v>
+      </c>
+      <c r="CH124" t="str">
+        <f t="shared" si="326"/>
+        <v>00</v>
+      </c>
+      <c r="CI124" t="str">
+        <f t="shared" si="303"/>
+        <v>01</v>
+      </c>
+      <c r="CJ124" t="str">
+        <f t="shared" si="304"/>
+        <v>07</v>
+      </c>
+      <c r="CK124" t="str">
+        <f t="shared" si="305"/>
+        <v>02</v>
+      </c>
+      <c r="CL124" t="str">
+        <f t="shared" si="306"/>
+        <v>03</v>
+      </c>
+      <c r="CM124" t="str">
+        <f t="shared" si="307"/>
+        <v>00</v>
+      </c>
+      <c r="CN124" t="str">
+        <f t="shared" si="308"/>
+        <v>00</v>
+      </c>
+      <c r="CO124" t="str">
+        <f t="shared" si="309"/>
+        <v>00</v>
+      </c>
+      <c r="CP124" t="str">
+        <f t="shared" si="310"/>
+        <v>00</v>
+      </c>
+      <c r="CQ124" t="str">
+        <f t="shared" si="311"/>
+        <v>00</v>
+      </c>
+      <c r="CR124" t="str">
+        <f t="shared" si="312"/>
+        <v>00</v>
+      </c>
+      <c r="CS124" t="str">
+        <f t="shared" si="313"/>
+        <v>00</v>
+      </c>
+      <c r="CT124" t="str">
+        <f t="shared" si="314"/>
+        <v>00</v>
+      </c>
+      <c r="CU124" t="str">
+        <f t="shared" si="315"/>
+        <v>00</v>
+      </c>
+      <c r="CV124" t="str">
+        <f t="shared" si="316"/>
+        <v>00</v>
+      </c>
+      <c r="CW124" t="str">
+        <f t="shared" si="317"/>
+        <v>00</v>
+      </c>
+      <c r="CX124" t="str">
+        <f t="shared" si="318"/>
+        <v>00</v>
+      </c>
+      <c r="CY124" t="str">
+        <f t="shared" si="319"/>
+        <v>00</v>
+      </c>
+      <c r="CZ124" t="str">
+        <f t="shared" si="320"/>
+        <v>00</v>
+      </c>
+      <c r="DA124" t="str">
+        <f t="shared" si="321"/>
+        <v>00</v>
+      </c>
+      <c r="DB124" t="str">
+        <f t="shared" si="322"/>
+        <v>04</v>
+      </c>
+      <c r="DC124" t="str">
+        <f t="shared" si="323"/>
+        <v>0107020300000000000000000000000000000004</v>
+      </c>
+      <c r="DD124" t="str">
+        <f t="shared" si="324"/>
+        <v>Active Sessions</v>
+      </c>
+      <c r="DE124" t="s">
+        <v>246</v>
+      </c>
+      <c r="DF124" t="s">
+        <v>223</v>
+      </c>
+      <c r="DG124" t="s">
+        <v>224</v>
+      </c>
+      <c r="DH124" t="s">
+        <v>225</v>
+      </c>
+      <c r="DI124" t="s">
+        <v>226</v>
+      </c>
+      <c r="DJ124" t="s">
+        <v>227</v>
+      </c>
+      <c r="DK124" t="s">
+        <v>228</v>
+      </c>
+      <c r="DL124" t="str">
+        <f t="shared" si="325"/>
+        <v>112,00,00,00,01,07,02,03,00,00,00,00,00,00,00,00,00,00,00,00,00,00,00,04,0107020300000000000000000000000000000004,Active Sessions,file112,Blk1,Blk2,Blk3,Blk4,Blk5,Blk6</v>
+      </c>
+    </row>
+    <row r="125" spans="2:116" x14ac:dyDescent="0.25">
+      <c r="B125">
+        <f t="shared" si="205"/>
+        <v>113</v>
+      </c>
+      <c r="F125" t="s">
+        <v>241</v>
+      </c>
+      <c r="W125">
+        <f t="shared" si="244"/>
+        <v>0</v>
+      </c>
+      <c r="X125">
+        <f t="shared" si="245"/>
+        <v>0</v>
+      </c>
+      <c r="Y125">
+        <f t="shared" si="246"/>
+        <v>0</v>
+      </c>
+      <c r="Z125">
+        <f t="shared" si="247"/>
+        <v>1</v>
+      </c>
+      <c r="AA125">
+        <f t="shared" si="248"/>
+        <v>0</v>
+      </c>
+      <c r="AB125">
+        <f t="shared" si="249"/>
+        <v>0</v>
+      </c>
+      <c r="AC125">
+        <f t="shared" si="250"/>
+        <v>0</v>
+      </c>
+      <c r="AD125">
+        <f t="shared" si="251"/>
+        <v>0</v>
+      </c>
+      <c r="AE125">
+        <f t="shared" si="252"/>
+        <v>0</v>
+      </c>
+      <c r="AF125">
+        <f t="shared" si="253"/>
+        <v>0</v>
+      </c>
+      <c r="AG125">
+        <f t="shared" si="254"/>
+        <v>0</v>
+      </c>
+      <c r="AH125">
+        <f t="shared" si="255"/>
+        <v>0</v>
+      </c>
+      <c r="AI125">
+        <f t="shared" si="256"/>
+        <v>0</v>
+      </c>
+      <c r="AJ125">
+        <f t="shared" si="257"/>
+        <v>0</v>
+      </c>
+      <c r="AK125">
+        <f t="shared" si="258"/>
+        <v>0</v>
+      </c>
+      <c r="AL125">
+        <f t="shared" si="259"/>
+        <v>0</v>
+      </c>
+      <c r="AM125">
+        <f t="shared" si="260"/>
+        <v>0</v>
+      </c>
+      <c r="AN125">
+        <f t="shared" si="261"/>
+        <v>0</v>
+      </c>
+      <c r="AO125">
+        <f t="shared" si="262"/>
+        <v>0</v>
+      </c>
+      <c r="AP125" s="2" t="str">
+        <f t="shared" si="263"/>
+        <v/>
+      </c>
+      <c r="AQ125" t="str">
+        <f t="shared" si="264"/>
+        <v>S</v>
+      </c>
+      <c r="AR125" t="str">
+        <f t="shared" si="265"/>
+        <v>S</v>
+      </c>
+      <c r="AS125" t="str">
+        <f t="shared" si="266"/>
+        <v>S</v>
+      </c>
+      <c r="AT125" t="str">
+        <f t="shared" si="267"/>
+        <v>+</v>
+      </c>
+      <c r="AU125" t="str">
+        <f t="shared" si="268"/>
+        <v/>
+      </c>
+      <c r="AV125" t="str">
+        <f t="shared" si="269"/>
+        <v/>
+      </c>
+      <c r="AW125" t="str">
+        <f t="shared" si="270"/>
+        <v/>
+      </c>
+      <c r="AX125" t="str">
+        <f t="shared" si="271"/>
+        <v/>
+      </c>
+      <c r="AY125" t="str">
+        <f t="shared" si="272"/>
+        <v/>
+      </c>
+      <c r="AZ125" t="str">
+        <f t="shared" si="273"/>
+        <v/>
+      </c>
+      <c r="BA125" t="str">
+        <f t="shared" si="274"/>
+        <v/>
+      </c>
+      <c r="BB125" t="str">
+        <f t="shared" si="275"/>
+        <v/>
+      </c>
+      <c r="BC125" t="str">
+        <f t="shared" si="276"/>
+        <v/>
+      </c>
+      <c r="BD125" t="str">
+        <f t="shared" si="277"/>
+        <v/>
+      </c>
+      <c r="BE125" t="str">
+        <f t="shared" si="278"/>
+        <v/>
+      </c>
+      <c r="BF125" t="str">
+        <f t="shared" si="279"/>
+        <v/>
+      </c>
+      <c r="BG125" t="str">
+        <f t="shared" si="280"/>
+        <v/>
+      </c>
+      <c r="BH125" t="str">
+        <f t="shared" si="281"/>
+        <v/>
+      </c>
+      <c r="BI125" t="str">
+        <f t="shared" si="282"/>
+        <v/>
+      </c>
+      <c r="BK125">
+        <f t="shared" si="283"/>
+        <v>1</v>
+      </c>
+      <c r="BL125">
+        <f t="shared" si="284"/>
+        <v>7</v>
+      </c>
+      <c r="BM125">
+        <f t="shared" si="285"/>
+        <v>2</v>
+      </c>
+      <c r="BN125">
+        <f t="shared" si="286"/>
+        <v>4</v>
+      </c>
+      <c r="BO125">
+        <f t="shared" si="287"/>
+        <v>0</v>
+      </c>
+      <c r="BP125">
+        <f t="shared" si="288"/>
+        <v>0</v>
+      </c>
+      <c r="BQ125">
+        <f t="shared" si="289"/>
+        <v>0</v>
+      </c>
+      <c r="BR125">
+        <f t="shared" si="290"/>
+        <v>0</v>
+      </c>
+      <c r="BS125">
+        <f t="shared" si="291"/>
+        <v>0</v>
+      </c>
+      <c r="BT125">
+        <f t="shared" si="292"/>
+        <v>0</v>
+      </c>
+      <c r="BU125">
+        <f t="shared" si="293"/>
+        <v>0</v>
+      </c>
+      <c r="BV125">
+        <f t="shared" si="294"/>
+        <v>0</v>
+      </c>
+      <c r="BW125">
+        <f t="shared" si="295"/>
+        <v>0</v>
+      </c>
+      <c r="BX125">
+        <f t="shared" si="296"/>
+        <v>0</v>
+      </c>
+      <c r="BY125">
+        <f t="shared" si="297"/>
+        <v>0</v>
+      </c>
+      <c r="BZ125">
+        <f t="shared" si="298"/>
+        <v>0</v>
+      </c>
+      <c r="CA125">
+        <f t="shared" si="299"/>
+        <v>0</v>
+      </c>
+      <c r="CB125">
+        <f t="shared" si="300"/>
+        <v>0</v>
+      </c>
+      <c r="CC125">
+        <f t="shared" si="301"/>
+        <v>0</v>
+      </c>
+      <c r="CE125" t="str">
+        <f t="shared" si="302"/>
+        <v>113</v>
+      </c>
+      <c r="CF125" t="str">
+        <f t="shared" si="326"/>
+        <v>00</v>
+      </c>
+      <c r="CG125" t="str">
+        <f t="shared" si="326"/>
+        <v>00</v>
+      </c>
+      <c r="CH125" t="str">
+        <f t="shared" si="326"/>
+        <v>00</v>
+      </c>
+      <c r="CI125" t="str">
+        <f t="shared" si="303"/>
+        <v>01</v>
+      </c>
+      <c r="CJ125" t="str">
+        <f t="shared" si="304"/>
+        <v>07</v>
+      </c>
+      <c r="CK125" t="str">
+        <f t="shared" si="305"/>
+        <v>02</v>
+      </c>
+      <c r="CL125" t="str">
+        <f t="shared" si="306"/>
+        <v>04</v>
+      </c>
+      <c r="CM125" t="str">
+        <f t="shared" si="307"/>
+        <v>00</v>
+      </c>
+      <c r="CN125" t="str">
+        <f t="shared" si="308"/>
+        <v>00</v>
+      </c>
+      <c r="CO125" t="str">
+        <f t="shared" si="309"/>
+        <v>00</v>
+      </c>
+      <c r="CP125" t="str">
+        <f t="shared" si="310"/>
+        <v>00</v>
+      </c>
+      <c r="CQ125" t="str">
+        <f t="shared" si="311"/>
+        <v>00</v>
+      </c>
+      <c r="CR125" t="str">
+        <f t="shared" si="312"/>
+        <v>00</v>
+      </c>
+      <c r="CS125" t="str">
+        <f t="shared" si="313"/>
+        <v>00</v>
+      </c>
+      <c r="CT125" t="str">
+        <f t="shared" si="314"/>
+        <v>00</v>
+      </c>
+      <c r="CU125" t="str">
+        <f t="shared" si="315"/>
+        <v>00</v>
+      </c>
+      <c r="CV125" t="str">
+        <f t="shared" si="316"/>
+        <v>00</v>
+      </c>
+      <c r="CW125" t="str">
+        <f t="shared" si="317"/>
+        <v>00</v>
+      </c>
+      <c r="CX125" t="str">
+        <f t="shared" si="318"/>
+        <v>00</v>
+      </c>
+      <c r="CY125" t="str">
+        <f t="shared" si="319"/>
+        <v>00</v>
+      </c>
+      <c r="CZ125" t="str">
+        <f t="shared" si="320"/>
+        <v>00</v>
+      </c>
+      <c r="DA125" t="str">
+        <f t="shared" si="321"/>
+        <v>00</v>
+      </c>
+      <c r="DB125" t="str">
+        <f t="shared" si="322"/>
+        <v>04</v>
+      </c>
+      <c r="DC125" t="str">
+        <f t="shared" si="323"/>
+        <v>0107020400000000000000000000000000000004</v>
+      </c>
+      <c r="DD125" t="str">
+        <f t="shared" si="324"/>
+        <v>Login History</v>
+      </c>
+      <c r="DE125" t="s">
+        <v>247</v>
+      </c>
+      <c r="DF125" t="s">
+        <v>223</v>
+      </c>
+      <c r="DG125" t="s">
+        <v>224</v>
+      </c>
+      <c r="DH125" t="s">
+        <v>225</v>
+      </c>
+      <c r="DI125" t="s">
+        <v>226</v>
+      </c>
+      <c r="DJ125" t="s">
+        <v>227</v>
+      </c>
+      <c r="DK125" t="s">
+        <v>228</v>
+      </c>
+      <c r="DL125" t="str">
+        <f t="shared" si="325"/>
+        <v>113,00,00,00,01,07,02,04,00,00,00,00,00,00,00,00,00,00,00,00,00,00,00,04,0107020400000000000000000000000000000004,Login History,file113,Blk1,Blk2,Blk3,Blk4,Blk5,Blk6</v>
+      </c>
+    </row>
+    <row r="126" spans="2:116" x14ac:dyDescent="0.25">
+      <c r="B126">
+        <f t="shared" si="205"/>
+        <v>114</v>
+      </c>
+      <c r="E126" t="s">
+        <v>16</v>
+      </c>
+      <c r="W126">
+        <f t="shared" si="244"/>
+        <v>0</v>
+      </c>
+      <c r="X126">
+        <f t="shared" si="245"/>
+        <v>0</v>
+      </c>
+      <c r="Y126">
+        <f t="shared" si="246"/>
+        <v>1</v>
+      </c>
+      <c r="Z126">
+        <f t="shared" si="247"/>
+        <v>0</v>
+      </c>
+      <c r="AA126">
+        <f t="shared" si="248"/>
+        <v>0</v>
+      </c>
+      <c r="AB126">
+        <f t="shared" si="249"/>
+        <v>0</v>
+      </c>
+      <c r="AC126">
+        <f t="shared" si="250"/>
+        <v>0</v>
+      </c>
+      <c r="AD126">
+        <f t="shared" si="251"/>
+        <v>0</v>
+      </c>
+      <c r="AE126">
+        <f t="shared" si="252"/>
+        <v>0</v>
+      </c>
+      <c r="AF126">
+        <f t="shared" si="253"/>
+        <v>0</v>
+      </c>
+      <c r="AG126">
+        <f t="shared" si="254"/>
+        <v>0</v>
+      </c>
+      <c r="AH126">
+        <f t="shared" si="255"/>
+        <v>0</v>
+      </c>
+      <c r="AI126">
+        <f t="shared" si="256"/>
+        <v>0</v>
+      </c>
+      <c r="AJ126">
+        <f t="shared" si="257"/>
+        <v>0</v>
+      </c>
+      <c r="AK126">
+        <f t="shared" si="258"/>
+        <v>0</v>
+      </c>
+      <c r="AL126">
+        <f t="shared" si="259"/>
+        <v>0</v>
+      </c>
+      <c r="AM126">
+        <f t="shared" si="260"/>
+        <v>0</v>
+      </c>
+      <c r="AN126">
+        <f t="shared" si="261"/>
+        <v>0</v>
+      </c>
+      <c r="AO126">
+        <f t="shared" si="262"/>
+        <v>0</v>
+      </c>
+      <c r="AP126" s="2" t="str">
+        <f t="shared" si="263"/>
+        <v/>
+      </c>
+      <c r="AQ126" t="str">
+        <f t="shared" si="264"/>
+        <v>S</v>
+      </c>
+      <c r="AR126" t="str">
+        <f t="shared" si="265"/>
+        <v>S</v>
+      </c>
+      <c r="AS126" t="str">
+        <f t="shared" si="266"/>
+        <v>+</v>
+      </c>
+      <c r="AT126" t="str">
+        <f t="shared" si="267"/>
+        <v/>
+      </c>
+      <c r="AU126" t="str">
+        <f t="shared" si="268"/>
+        <v/>
+      </c>
+      <c r="AV126" t="str">
+        <f t="shared" si="269"/>
+        <v/>
+      </c>
+      <c r="AW126" t="str">
+        <f t="shared" si="270"/>
+        <v/>
+      </c>
+      <c r="AX126" t="str">
+        <f t="shared" si="271"/>
+        <v/>
+      </c>
+      <c r="AY126" t="str">
+        <f t="shared" si="272"/>
+        <v/>
+      </c>
+      <c r="AZ126" t="str">
+        <f t="shared" si="273"/>
+        <v/>
+      </c>
+      <c r="BA126" t="str">
+        <f t="shared" si="274"/>
+        <v/>
+      </c>
+      <c r="BB126" t="str">
+        <f t="shared" si="275"/>
+        <v/>
+      </c>
+      <c r="BC126" t="str">
+        <f t="shared" si="276"/>
+        <v/>
+      </c>
+      <c r="BD126" t="str">
+        <f t="shared" si="277"/>
+        <v/>
+      </c>
+      <c r="BE126" t="str">
+        <f t="shared" si="278"/>
+        <v/>
+      </c>
+      <c r="BF126" t="str">
+        <f t="shared" si="279"/>
+        <v/>
+      </c>
+      <c r="BG126" t="str">
+        <f t="shared" si="280"/>
+        <v/>
+      </c>
+      <c r="BH126" t="str">
+        <f t="shared" si="281"/>
+        <v/>
+      </c>
+      <c r="BI126" t="str">
+        <f t="shared" si="282"/>
+        <v/>
+      </c>
+      <c r="BK126">
+        <f t="shared" si="283"/>
+        <v>1</v>
+      </c>
+      <c r="BL126">
+        <f t="shared" si="284"/>
+        <v>7</v>
+      </c>
+      <c r="BM126">
+        <f t="shared" si="285"/>
+        <v>3</v>
+      </c>
+      <c r="BN126">
+        <f t="shared" si="286"/>
+        <v>0</v>
+      </c>
+      <c r="BO126">
+        <f t="shared" si="287"/>
+        <v>0</v>
+      </c>
+      <c r="BP126">
+        <f t="shared" si="288"/>
+        <v>0</v>
+      </c>
+      <c r="BQ126">
+        <f t="shared" si="289"/>
+        <v>0</v>
+      </c>
+      <c r="BR126">
+        <f t="shared" si="290"/>
+        <v>0</v>
+      </c>
+      <c r="BS126">
+        <f t="shared" si="291"/>
+        <v>0</v>
+      </c>
+      <c r="BT126">
+        <f t="shared" si="292"/>
+        <v>0</v>
+      </c>
+      <c r="BU126">
+        <f t="shared" si="293"/>
+        <v>0</v>
+      </c>
+      <c r="BV126">
+        <f t="shared" si="294"/>
+        <v>0</v>
+      </c>
+      <c r="BW126">
+        <f t="shared" si="295"/>
+        <v>0</v>
+      </c>
+      <c r="BX126">
+        <f t="shared" si="296"/>
+        <v>0</v>
+      </c>
+      <c r="BY126">
+        <f t="shared" si="297"/>
+        <v>0</v>
+      </c>
+      <c r="BZ126">
+        <f t="shared" si="298"/>
+        <v>0</v>
+      </c>
+      <c r="CA126">
+        <f t="shared" si="299"/>
+        <v>0</v>
+      </c>
+      <c r="CB126">
+        <f t="shared" si="300"/>
+        <v>0</v>
+      </c>
+      <c r="CC126">
+        <f t="shared" si="301"/>
+        <v>0</v>
+      </c>
+      <c r="CE126" t="str">
+        <f t="shared" si="302"/>
+        <v>114</v>
+      </c>
+      <c r="CF126" t="str">
+        <f t="shared" si="326"/>
+        <v>00</v>
+      </c>
+      <c r="CG126" t="str">
+        <f t="shared" si="326"/>
+        <v>00</v>
+      </c>
+      <c r="CH126" t="str">
+        <f t="shared" si="326"/>
+        <v>00</v>
+      </c>
+      <c r="CI126" t="str">
+        <f t="shared" si="303"/>
+        <v>01</v>
+      </c>
+      <c r="CJ126" t="str">
+        <f t="shared" si="304"/>
+        <v>07</v>
+      </c>
+      <c r="CK126" t="str">
+        <f t="shared" si="305"/>
+        <v>03</v>
+      </c>
+      <c r="CL126" t="str">
+        <f t="shared" si="306"/>
+        <v>00</v>
+      </c>
+      <c r="CM126" t="str">
+        <f t="shared" si="307"/>
+        <v>00</v>
+      </c>
+      <c r="CN126" t="str">
+        <f t="shared" si="308"/>
+        <v>00</v>
+      </c>
+      <c r="CO126" t="str">
+        <f t="shared" si="309"/>
+        <v>00</v>
+      </c>
+      <c r="CP126" t="str">
+        <f t="shared" si="310"/>
+        <v>00</v>
+      </c>
+      <c r="CQ126" t="str">
+        <f t="shared" si="311"/>
+        <v>00</v>
+      </c>
+      <c r="CR126" t="str">
+        <f t="shared" si="312"/>
+        <v>00</v>
+      </c>
+      <c r="CS126" t="str">
+        <f t="shared" si="313"/>
+        <v>00</v>
+      </c>
+      <c r="CT126" t="str">
+        <f t="shared" si="314"/>
+        <v>00</v>
+      </c>
+      <c r="CU126" t="str">
+        <f t="shared" si="315"/>
+        <v>00</v>
+      </c>
+      <c r="CV126" t="str">
+        <f t="shared" si="316"/>
+        <v>00</v>
+      </c>
+      <c r="CW126" t="str">
+        <f t="shared" si="317"/>
+        <v>00</v>
+      </c>
+      <c r="CX126" t="str">
+        <f t="shared" si="318"/>
+        <v>00</v>
+      </c>
+      <c r="CY126" t="str">
+        <f t="shared" si="319"/>
+        <v>00</v>
+      </c>
+      <c r="CZ126" t="str">
+        <f t="shared" si="320"/>
+        <v>00</v>
+      </c>
+      <c r="DA126" t="str">
+        <f t="shared" si="321"/>
+        <v>00</v>
+      </c>
+      <c r="DB126" t="str">
+        <f t="shared" si="322"/>
+        <v>03</v>
+      </c>
+      <c r="DC126" t="str">
+        <f t="shared" si="323"/>
+        <v>0107030000000000000000000000000000000003</v>
+      </c>
+      <c r="DD126" t="str">
+        <f t="shared" si="324"/>
+        <v>Notification</v>
+      </c>
+      <c r="DE126" t="s">
+        <v>248</v>
+      </c>
+      <c r="DF126" t="s">
+        <v>223</v>
+      </c>
+      <c r="DG126" t="s">
+        <v>224</v>
+      </c>
+      <c r="DH126" t="s">
+        <v>225</v>
+      </c>
+      <c r="DI126" t="s">
+        <v>226</v>
+      </c>
+      <c r="DJ126" t="s">
+        <v>227</v>
+      </c>
+      <c r="DK126" t="s">
+        <v>228</v>
+      </c>
+      <c r="DL126" t="str">
+        <f t="shared" si="325"/>
+        <v>114,00,00,00,01,07,03,00,00,00,00,00,00,00,00,00,00,00,00,00,00,00,00,03,0107030000000000000000000000000000000003,Notification,file114,Blk1,Blk2,Blk3,Blk4,Blk5,Blk6</v>
+      </c>
+    </row>
+    <row r="127" spans="2:116" x14ac:dyDescent="0.25">
+      <c r="B127">
+        <f t="shared" si="205"/>
+        <v>115</v>
+      </c>
+      <c r="E127" t="s">
+        <v>236</v>
+      </c>
+      <c r="W127">
+        <f t="shared" si="244"/>
+        <v>0</v>
+      </c>
+      <c r="X127">
+        <f t="shared" si="245"/>
+        <v>0</v>
+      </c>
+      <c r="Y127">
+        <f t="shared" si="246"/>
+        <v>1</v>
+      </c>
+      <c r="Z127">
+        <f t="shared" si="247"/>
+        <v>0</v>
+      </c>
+      <c r="AA127">
+        <f t="shared" si="248"/>
+        <v>0</v>
+      </c>
+      <c r="AB127">
+        <f t="shared" si="249"/>
+        <v>0</v>
+      </c>
+      <c r="AC127">
+        <f t="shared" si="250"/>
+        <v>0</v>
+      </c>
+      <c r="AD127">
+        <f t="shared" si="251"/>
+        <v>0</v>
+      </c>
+      <c r="AE127">
+        <f t="shared" si="252"/>
+        <v>0</v>
+      </c>
+      <c r="AF127">
+        <f t="shared" si="253"/>
+        <v>0</v>
+      </c>
+      <c r="AG127">
+        <f t="shared" si="254"/>
+        <v>0</v>
+      </c>
+      <c r="AH127">
+        <f t="shared" si="255"/>
+        <v>0</v>
+      </c>
+      <c r="AI127">
+        <f t="shared" si="256"/>
+        <v>0</v>
+      </c>
+      <c r="AJ127">
+        <f t="shared" si="257"/>
+        <v>0</v>
+      </c>
+      <c r="AK127">
+        <f t="shared" si="258"/>
+        <v>0</v>
+      </c>
+      <c r="AL127">
+        <f t="shared" si="259"/>
+        <v>0</v>
+      </c>
+      <c r="AM127">
+        <f t="shared" si="260"/>
+        <v>0</v>
+      </c>
+      <c r="AN127">
+        <f t="shared" si="261"/>
+        <v>0</v>
+      </c>
+      <c r="AO127">
+        <f t="shared" si="262"/>
+        <v>0</v>
+      </c>
+      <c r="AP127" s="2" t="str">
+        <f t="shared" si="263"/>
+        <v/>
+      </c>
+      <c r="AQ127" t="str">
+        <f t="shared" si="264"/>
+        <v>S</v>
+      </c>
+      <c r="AR127" t="str">
+        <f t="shared" si="265"/>
+        <v>S</v>
+      </c>
+      <c r="AS127" t="str">
+        <f t="shared" si="266"/>
+        <v>+</v>
+      </c>
+      <c r="AT127" t="str">
+        <f t="shared" si="267"/>
+        <v/>
+      </c>
+      <c r="AU127" t="str">
+        <f t="shared" si="268"/>
+        <v/>
+      </c>
+      <c r="AV127" t="str">
+        <f t="shared" si="269"/>
+        <v/>
+      </c>
+      <c r="AW127" t="str">
+        <f t="shared" si="270"/>
+        <v/>
+      </c>
+      <c r="AX127" t="str">
+        <f t="shared" si="271"/>
+        <v/>
+      </c>
+      <c r="AY127" t="str">
+        <f t="shared" si="272"/>
+        <v/>
+      </c>
+      <c r="AZ127" t="str">
+        <f t="shared" si="273"/>
+        <v/>
+      </c>
+      <c r="BA127" t="str">
+        <f t="shared" si="274"/>
+        <v/>
+      </c>
+      <c r="BB127" t="str">
+        <f t="shared" si="275"/>
+        <v/>
+      </c>
+      <c r="BC127" t="str">
+        <f t="shared" si="276"/>
+        <v/>
+      </c>
+      <c r="BD127" t="str">
+        <f t="shared" si="277"/>
+        <v/>
+      </c>
+      <c r="BE127" t="str">
+        <f t="shared" si="278"/>
+        <v/>
+      </c>
+      <c r="BF127" t="str">
+        <f t="shared" si="279"/>
+        <v/>
+      </c>
+      <c r="BG127" t="str">
+        <f t="shared" si="280"/>
+        <v/>
+      </c>
+      <c r="BH127" t="str">
+        <f t="shared" si="281"/>
+        <v/>
+      </c>
+      <c r="BI127" t="str">
+        <f t="shared" si="282"/>
+        <v/>
+      </c>
+      <c r="BK127">
+        <f t="shared" si="283"/>
+        <v>1</v>
+      </c>
+      <c r="BL127">
+        <f t="shared" si="284"/>
+        <v>7</v>
+      </c>
+      <c r="BM127">
+        <f t="shared" si="285"/>
+        <v>4</v>
+      </c>
+      <c r="BN127">
+        <f t="shared" si="286"/>
+        <v>0</v>
+      </c>
+      <c r="BO127">
+        <f t="shared" si="287"/>
+        <v>0</v>
+      </c>
+      <c r="BP127">
+        <f t="shared" si="288"/>
+        <v>0</v>
+      </c>
+      <c r="BQ127">
+        <f t="shared" si="289"/>
+        <v>0</v>
+      </c>
+      <c r="BR127">
+        <f t="shared" si="290"/>
+        <v>0</v>
+      </c>
+      <c r="BS127">
+        <f t="shared" si="291"/>
+        <v>0</v>
+      </c>
+      <c r="BT127">
+        <f t="shared" si="292"/>
+        <v>0</v>
+      </c>
+      <c r="BU127">
+        <f t="shared" si="293"/>
+        <v>0</v>
+      </c>
+      <c r="BV127">
+        <f t="shared" si="294"/>
+        <v>0</v>
+      </c>
+      <c r="BW127">
+        <f t="shared" si="295"/>
+        <v>0</v>
+      </c>
+      <c r="BX127">
+        <f t="shared" si="296"/>
+        <v>0</v>
+      </c>
+      <c r="BY127">
+        <f t="shared" si="297"/>
+        <v>0</v>
+      </c>
+      <c r="BZ127">
+        <f t="shared" si="298"/>
+        <v>0</v>
+      </c>
+      <c r="CA127">
+        <f t="shared" si="299"/>
+        <v>0</v>
+      </c>
+      <c r="CB127">
+        <f t="shared" si="300"/>
+        <v>0</v>
+      </c>
+      <c r="CC127">
+        <f t="shared" si="301"/>
+        <v>0</v>
+      </c>
+      <c r="CE127" t="str">
+        <f t="shared" si="302"/>
+        <v>115</v>
+      </c>
+      <c r="CF127" t="str">
+        <f t="shared" si="326"/>
+        <v>00</v>
+      </c>
+      <c r="CG127" t="str">
+        <f t="shared" si="326"/>
+        <v>00</v>
+      </c>
+      <c r="CH127" t="str">
+        <f t="shared" si="326"/>
+        <v>00</v>
+      </c>
+      <c r="CI127" t="str">
+        <f t="shared" si="303"/>
+        <v>01</v>
+      </c>
+      <c r="CJ127" t="str">
+        <f t="shared" si="304"/>
+        <v>07</v>
+      </c>
+      <c r="CK127" t="str">
+        <f t="shared" si="305"/>
+        <v>04</v>
+      </c>
+      <c r="CL127" t="str">
+        <f t="shared" si="306"/>
+        <v>00</v>
+      </c>
+      <c r="CM127" t="str">
+        <f t="shared" si="307"/>
+        <v>00</v>
+      </c>
+      <c r="CN127" t="str">
+        <f t="shared" si="308"/>
+        <v>00</v>
+      </c>
+      <c r="CO127" t="str">
+        <f t="shared" si="309"/>
+        <v>00</v>
+      </c>
+      <c r="CP127" t="str">
+        <f t="shared" si="310"/>
+        <v>00</v>
+      </c>
+      <c r="CQ127" t="str">
+        <f t="shared" si="311"/>
+        <v>00</v>
+      </c>
+      <c r="CR127" t="str">
+        <f t="shared" si="312"/>
+        <v>00</v>
+      </c>
+      <c r="CS127" t="str">
+        <f t="shared" si="313"/>
+        <v>00</v>
+      </c>
+      <c r="CT127" t="str">
+        <f t="shared" si="314"/>
+        <v>00</v>
+      </c>
+      <c r="CU127" t="str">
+        <f t="shared" si="315"/>
+        <v>00</v>
+      </c>
+      <c r="CV127" t="str">
+        <f t="shared" si="316"/>
+        <v>00</v>
+      </c>
+      <c r="CW127" t="str">
+        <f t="shared" si="317"/>
+        <v>00</v>
+      </c>
+      <c r="CX127" t="str">
+        <f t="shared" si="318"/>
+        <v>00</v>
+      </c>
+      <c r="CY127" t="str">
+        <f t="shared" si="319"/>
+        <v>00</v>
+      </c>
+      <c r="CZ127" t="str">
+        <f t="shared" si="320"/>
+        <v>00</v>
+      </c>
+      <c r="DA127" t="str">
+        <f t="shared" si="321"/>
+        <v>00</v>
+      </c>
+      <c r="DB127" t="str">
+        <f t="shared" si="322"/>
+        <v>03</v>
+      </c>
+      <c r="DC127" t="str">
+        <f t="shared" ref="DC127:DC128" si="327">_xlfn.CONCAT(CI127:DB127)</f>
+        <v>0107040000000000000000000000000000000003</v>
+      </c>
+      <c r="DD127" t="str">
+        <f t="shared" ref="DD127:DD128" si="328">_xlfn.CONCAT(C127:U127)</f>
+        <v>Privacy</v>
+      </c>
+      <c r="DE127" t="s">
+        <v>249</v>
+      </c>
+      <c r="DF127" t="s">
+        <v>223</v>
+      </c>
+      <c r="DG127" t="s">
+        <v>224</v>
+      </c>
+      <c r="DH127" t="s">
+        <v>225</v>
+      </c>
+      <c r="DI127" t="s">
+        <v>226</v>
+      </c>
+      <c r="DJ127" t="s">
+        <v>227</v>
+      </c>
+      <c r="DK127" t="s">
+        <v>228</v>
+      </c>
+      <c r="DL127" t="str">
+        <f t="shared" ref="DL127:DL128" si="329">_xlfn.TEXTJOIN(",", TRUE,CE127:DK127)</f>
+        <v>115,00,00,00,01,07,04,00,00,00,00,00,00,00,00,00,00,00,00,00,00,00,00,03,0107040000000000000000000000000000000003,Privacy,file115,Blk1,Blk2,Blk3,Blk4,Blk5,Blk6</v>
+      </c>
+    </row>
+    <row r="128" spans="2:116" x14ac:dyDescent="0.25">
+      <c r="B128">
+        <f t="shared" si="205"/>
+        <v>116</v>
+      </c>
+      <c r="E128" t="s">
+        <v>237</v>
+      </c>
+      <c r="W128">
+        <f t="shared" si="244"/>
+        <v>0</v>
+      </c>
+      <c r="X128">
+        <f t="shared" si="245"/>
+        <v>0</v>
+      </c>
+      <c r="Y128">
+        <f t="shared" si="246"/>
+        <v>1</v>
+      </c>
+      <c r="Z128">
+        <f t="shared" si="247"/>
+        <v>0</v>
+      </c>
+      <c r="AA128">
+        <f t="shared" si="248"/>
+        <v>0</v>
+      </c>
+      <c r="AB128">
+        <f t="shared" si="249"/>
+        <v>0</v>
+      </c>
+      <c r="AC128">
+        <f t="shared" si="250"/>
+        <v>0</v>
+      </c>
+      <c r="AD128">
+        <f t="shared" si="251"/>
+        <v>0</v>
+      </c>
+      <c r="AE128">
+        <f t="shared" si="252"/>
+        <v>0</v>
+      </c>
+      <c r="AF128">
+        <f t="shared" si="253"/>
+        <v>0</v>
+      </c>
+      <c r="AG128">
+        <f t="shared" si="254"/>
+        <v>0</v>
+      </c>
+      <c r="AH128">
+        <f t="shared" si="255"/>
+        <v>0</v>
+      </c>
+      <c r="AI128">
+        <f t="shared" si="256"/>
+        <v>0</v>
+      </c>
+      <c r="AJ128">
+        <f t="shared" si="257"/>
+        <v>0</v>
+      </c>
+      <c r="AK128">
+        <f t="shared" si="258"/>
+        <v>0</v>
+      </c>
+      <c r="AL128">
+        <f t="shared" si="259"/>
+        <v>0</v>
+      </c>
+      <c r="AM128">
+        <f t="shared" si="260"/>
+        <v>0</v>
+      </c>
+      <c r="AN128">
+        <f t="shared" si="261"/>
+        <v>0</v>
+      </c>
+      <c r="AO128">
+        <f t="shared" si="262"/>
+        <v>0</v>
+      </c>
+      <c r="AP128" s="2" t="str">
+        <f t="shared" si="263"/>
+        <v/>
+      </c>
+      <c r="AQ128" t="str">
+        <f t="shared" si="264"/>
+        <v>S</v>
+      </c>
+      <c r="AR128" t="str">
+        <f t="shared" si="265"/>
+        <v>S</v>
+      </c>
+      <c r="AS128" t="str">
+        <f t="shared" si="266"/>
+        <v>+</v>
+      </c>
+      <c r="AT128" t="str">
+        <f t="shared" si="267"/>
+        <v/>
+      </c>
+      <c r="AU128" t="str">
+        <f t="shared" si="268"/>
+        <v/>
+      </c>
+      <c r="AV128" t="str">
+        <f t="shared" si="269"/>
+        <v/>
+      </c>
+      <c r="AW128" t="str">
+        <f t="shared" si="270"/>
+        <v/>
+      </c>
+      <c r="AX128" t="str">
+        <f t="shared" si="271"/>
+        <v/>
+      </c>
+      <c r="AY128" t="str">
+        <f t="shared" si="272"/>
+        <v/>
+      </c>
+      <c r="AZ128" t="str">
+        <f t="shared" si="273"/>
+        <v/>
+      </c>
+      <c r="BA128" t="str">
+        <f t="shared" si="274"/>
+        <v/>
+      </c>
+      <c r="BB128" t="str">
+        <f t="shared" si="275"/>
+        <v/>
+      </c>
+      <c r="BC128" t="str">
+        <f t="shared" si="276"/>
+        <v/>
+      </c>
+      <c r="BD128" t="str">
+        <f t="shared" si="277"/>
+        <v/>
+      </c>
+      <c r="BE128" t="str">
+        <f t="shared" si="278"/>
+        <v/>
+      </c>
+      <c r="BF128" t="str">
+        <f t="shared" si="279"/>
+        <v/>
+      </c>
+      <c r="BG128" t="str">
+        <f t="shared" si="280"/>
+        <v/>
+      </c>
+      <c r="BH128" t="str">
+        <f t="shared" si="281"/>
+        <v/>
+      </c>
+      <c r="BI128" t="str">
+        <f t="shared" si="282"/>
+        <v/>
+      </c>
+      <c r="BK128">
+        <f t="shared" si="283"/>
+        <v>1</v>
+      </c>
+      <c r="BL128">
+        <f t="shared" si="284"/>
+        <v>7</v>
+      </c>
+      <c r="BM128">
+        <f t="shared" si="285"/>
+        <v>5</v>
+      </c>
+      <c r="BN128">
+        <f t="shared" si="286"/>
+        <v>0</v>
+      </c>
+      <c r="BO128">
+        <f t="shared" si="287"/>
+        <v>0</v>
+      </c>
+      <c r="BP128">
+        <f t="shared" si="288"/>
+        <v>0</v>
+      </c>
+      <c r="BQ128">
+        <f t="shared" si="289"/>
+        <v>0</v>
+      </c>
+      <c r="BR128">
+        <f t="shared" si="290"/>
+        <v>0</v>
+      </c>
+      <c r="BS128">
+        <f t="shared" si="291"/>
+        <v>0</v>
+      </c>
+      <c r="BT128">
+        <f t="shared" si="292"/>
+        <v>0</v>
+      </c>
+      <c r="BU128">
+        <f t="shared" si="293"/>
+        <v>0</v>
+      </c>
+      <c r="BV128">
+        <f t="shared" si="294"/>
+        <v>0</v>
+      </c>
+      <c r="BW128">
+        <f t="shared" si="295"/>
+        <v>0</v>
+      </c>
+      <c r="BX128">
+        <f t="shared" si="296"/>
+        <v>0</v>
+      </c>
+      <c r="BY128">
+        <f t="shared" si="297"/>
+        <v>0</v>
+      </c>
+      <c r="BZ128">
+        <f t="shared" si="298"/>
+        <v>0</v>
+      </c>
+      <c r="CA128">
+        <f t="shared" si="299"/>
+        <v>0</v>
+      </c>
+      <c r="CB128">
+        <f t="shared" si="300"/>
+        <v>0</v>
+      </c>
+      <c r="CC128">
+        <f t="shared" si="301"/>
+        <v>0</v>
+      </c>
+      <c r="CE128" t="str">
+        <f t="shared" si="302"/>
+        <v>116</v>
+      </c>
+      <c r="CF128" t="str">
+        <f t="shared" si="326"/>
+        <v>00</v>
+      </c>
+      <c r="CG128" t="str">
+        <f t="shared" si="326"/>
+        <v>00</v>
+      </c>
+      <c r="CH128" t="str">
+        <f t="shared" si="326"/>
+        <v>00</v>
+      </c>
+      <c r="CI128" t="str">
+        <f t="shared" si="303"/>
+        <v>01</v>
+      </c>
+      <c r="CJ128" t="str">
+        <f t="shared" si="304"/>
+        <v>07</v>
+      </c>
+      <c r="CK128" t="str">
+        <f t="shared" si="305"/>
+        <v>05</v>
+      </c>
+      <c r="CL128" t="str">
+        <f t="shared" si="306"/>
+        <v>00</v>
+      </c>
+      <c r="CM128" t="str">
+        <f t="shared" si="307"/>
+        <v>00</v>
+      </c>
+      <c r="CN128" t="str">
+        <f t="shared" si="308"/>
+        <v>00</v>
+      </c>
+      <c r="CO128" t="str">
+        <f t="shared" si="309"/>
+        <v>00</v>
+      </c>
+      <c r="CP128" t="str">
+        <f t="shared" si="310"/>
+        <v>00</v>
+      </c>
+      <c r="CQ128" t="str">
+        <f t="shared" si="311"/>
+        <v>00</v>
+      </c>
+      <c r="CR128" t="str">
+        <f t="shared" si="312"/>
+        <v>00</v>
+      </c>
+      <c r="CS128" t="str">
+        <f t="shared" si="313"/>
+        <v>00</v>
+      </c>
+      <c r="CT128" t="str">
+        <f t="shared" si="314"/>
+        <v>00</v>
+      </c>
+      <c r="CU128" t="str">
+        <f t="shared" si="315"/>
+        <v>00</v>
+      </c>
+      <c r="CV128" t="str">
+        <f t="shared" si="316"/>
+        <v>00</v>
+      </c>
+      <c r="CW128" t="str">
+        <f t="shared" si="317"/>
+        <v>00</v>
+      </c>
+      <c r="CX128" t="str">
+        <f t="shared" si="318"/>
+        <v>00</v>
+      </c>
+      <c r="CY128" t="str">
+        <f t="shared" si="319"/>
+        <v>00</v>
+      </c>
+      <c r="CZ128" t="str">
+        <f t="shared" si="320"/>
+        <v>00</v>
+      </c>
+      <c r="DA128" t="str">
+        <f t="shared" si="321"/>
+        <v>00</v>
+      </c>
+      <c r="DB128" t="str">
+        <f t="shared" si="322"/>
+        <v>03</v>
+      </c>
+      <c r="DC128" t="str">
+        <f t="shared" si="327"/>
+        <v>0107050000000000000000000000000000000003</v>
+      </c>
+      <c r="DD128" t="str">
+        <f t="shared" si="328"/>
+        <v>Account</v>
+      </c>
+      <c r="DE128" t="s">
+        <v>250</v>
+      </c>
+      <c r="DF128" t="s">
+        <v>223</v>
+      </c>
+      <c r="DG128" t="s">
+        <v>224</v>
+      </c>
+      <c r="DH128" t="s">
+        <v>225</v>
+      </c>
+      <c r="DI128" t="s">
+        <v>226</v>
+      </c>
+      <c r="DJ128" t="s">
+        <v>227</v>
+      </c>
+      <c r="DK128" t="s">
+        <v>228</v>
+      </c>
+      <c r="DL128" t="str">
+        <f t="shared" si="329"/>
+        <v>116,00,00,00,01,07,05,00,00,00,00,00,00,00,00,00,00,00,00,00,00,00,00,03,0107050000000000000000000000000000000003,Account,file116,Blk1,Blk2,Blk3,Blk4,Blk5,Blk6</v>
       </c>
     </row>
   </sheetData>
@@ -40846,6 +44603,7 @@
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>